<commit_message>
Reviewed and edited the bom
</commit_message>
<xml_diff>
--- a/bom.csv.xlsx
+++ b/bom.csv.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10928"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alisruzh\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/logancalder/Documents/Aquatonomous/Aqua BMS Monitor/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{D98C1871-A47A-42AA-AAE5-9A254DA12573}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32458A0D-0D7E-3148-9764-14C898564C45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{EA634A8A-7489-4C3E-A3E3-2BEB5E00DD22}"/>
+    <workbookView xWindow="16540" yWindow="780" windowWidth="13700" windowHeight="17860" xr2:uid="{EA634A8A-7489-4C3E-A3E3-2BEB5E00DD22}"/>
   </bookViews>
   <sheets>
     <sheet name="bom" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="467" uniqueCount="377">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="569" uniqueCount="407">
   <si>
     <t>Designator</t>
   </si>
@@ -142,9 +142,6 @@
     <t>BR1</t>
   </si>
   <si>
-    <t>C14675</t>
-  </si>
-  <si>
     <t>C70, C71, C72, MCUC18</t>
   </si>
   <si>
@@ -589,9 +586,6 @@
     <t>200_R1210</t>
   </si>
   <si>
-    <t>C26060</t>
-  </si>
-  <si>
     <t>S1</t>
   </si>
   <si>
@@ -1066,9 +1060,6 @@
     <t>LTC4359-DCB</t>
   </si>
   <si>
-    <t>505-LTC4359CDCB#TRPBFCT-ND</t>
-  </si>
-  <si>
     <t>U9</t>
   </si>
   <si>
@@ -1151,13 +1142,112 @@
   </si>
   <si>
     <t>C5123609</t>
+  </si>
+  <si>
+    <t>Logan Flag</t>
+  </si>
+  <si>
+    <t>x</t>
+  </si>
+  <si>
+    <t>C177347</t>
+  </si>
+  <si>
+    <t>Switched</t>
+  </si>
+  <si>
+    <t>Comments</t>
+  </si>
+  <si>
+    <t>Somehow</t>
+  </si>
+  <si>
+    <t>16V, but that's okay!</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t>Validated by Logan</t>
+  </si>
+  <si>
+    <t>wrong value originally</t>
+  </si>
+  <si>
+    <t>Polarity -&gt; should make sure assigned properly</t>
+  </si>
+  <si>
+    <t>Throughhole - we can just order</t>
+  </si>
+  <si>
+    <t>C320558</t>
+  </si>
+  <si>
+    <t>Found a new tvs diode</t>
+  </si>
+  <si>
+    <t>C1973936</t>
+  </si>
+  <si>
+    <t>Found a new tvs diode - supposeely compatable with the DO-219AB package</t>
+  </si>
+  <si>
+    <t>great deal - keep pcba</t>
+  </si>
+  <si>
+    <t>This doesn't need to be PCBA - ungodly cheap tho</t>
+  </si>
+  <si>
+    <t>This doesn't need to be pcba and is smt we should buy anyway</t>
+  </si>
+  <si>
+    <t>Alisa, please double check this just cause it's complex. But looks fine</t>
+  </si>
+  <si>
+    <t>not 100% sure, but pre sure this is right</t>
+  </si>
+  <si>
+    <t>This is fine, but supposedly the same footprint as the pmos, but they look different</t>
+  </si>
+  <si>
+    <t>was - C26060 which is wrong</t>
+  </si>
+  <si>
+    <t>C102427</t>
+  </si>
+  <si>
+    <t>Throughpin all good to ignore from JLC</t>
+  </si>
+  <si>
+    <t>Not an amazing deal could do non-JLC</t>
+  </si>
+  <si>
+    <t>C4350330</t>
+  </si>
+  <si>
+    <t>Blank - Added by logan</t>
+  </si>
+  <si>
+    <t>Blank -Added by logan</t>
+  </si>
+  <si>
+    <t>Through pin and we don't necessairly want them right in the board - I would not have them assembled on board</t>
+  </si>
+  <si>
+    <t>THANK GOD THEY HAVE THIS</t>
+  </si>
+  <si>
+    <t>C7454463</t>
+  </si>
+  <si>
+    <t>I think this is the right one, pls double check505-LTC4359CDCB#TRPBFCT-ND</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1290,6 +1380,13 @@
       <color theme="0"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -1634,10 +1731,17 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="42">
@@ -2014,18 +2118,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2EF7A2F2-D173-446E-BAD3-537DE2CE4F10}">
-  <dimension ref="A1:F139"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:J139"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="60.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="38.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="60.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="38.83203125" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="7.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="23.77734375" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="23.83203125" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="10.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="28.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="28.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="22.6640625" style="4" customWidth="1"/>
+    <col min="9" max="9" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2044,8 +2150,17 @@
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G1" s="1" t="s">
+        <v>374</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>378</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>6</v>
       </c>
@@ -2061,8 +2176,14 @@
       <c r="E2" s="1" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="H2" s="4" t="s">
+        <v>379</v>
+      </c>
+      <c r="I2" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>10</v>
       </c>
@@ -2078,8 +2199,11 @@
       <c r="E3" s="1" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="I3" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>14</v>
       </c>
@@ -2095,8 +2219,11 @@
       <c r="E4" s="1" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="I4" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>18</v>
       </c>
@@ -2112,8 +2239,11 @@
       <c r="E5" s="1" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="I5" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>21</v>
       </c>
@@ -2129,8 +2259,14 @@
       <c r="E6" s="1" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="H6" s="4" t="s">
+        <v>384</v>
+      </c>
+      <c r="I6" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>25</v>
       </c>
@@ -2146,8 +2282,14 @@
       <c r="F7" s="1" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G7" s="1" t="s">
+        <v>375</v>
+      </c>
+      <c r="H7" s="4" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
         <v>29</v>
       </c>
@@ -2163,8 +2305,11 @@
       <c r="E8" s="1" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="I8" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
         <v>32</v>
       </c>
@@ -2180,8 +2325,11 @@
       <c r="E9" s="1" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="I9" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>36</v>
       </c>
@@ -2197,8 +2345,11 @@
       <c r="E10" s="1" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="I10" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
         <v>39</v>
       </c>
@@ -2212,46 +2363,67 @@
         <v>100</v>
       </c>
       <c r="E11" s="1" t="s">
+        <v>376</v>
+      </c>
+      <c r="G11" t="s">
+        <v>375</v>
+      </c>
+      <c r="H11" s="4" t="s">
+        <v>383</v>
+      </c>
+      <c r="I11" s="1" t="s">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+      <c r="A12" s="1" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A12" s="1" t="s">
+      <c r="B12" s="1" t="s">
         <v>41</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>42</v>
       </c>
       <c r="C12" s="1">
         <v>4</v>
       </c>
       <c r="D12" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="E12" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="E12" s="1" t="s">
+      <c r="H12" s="4" t="s">
+        <v>380</v>
+      </c>
+      <c r="I12" s="1" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" ht="32" x14ac:dyDescent="0.2">
+      <c r="A13" s="1" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A13" s="1" t="s">
+      <c r="B13" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="B13" s="1" t="s">
+      <c r="C13" s="1">
+        <v>1</v>
+      </c>
+      <c r="D13" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="C13" s="1">
-        <v>1</v>
-      </c>
-      <c r="D13" s="1" t="s">
+      <c r="E13" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="E13" s="1" t="s">
+      <c r="G13" s="1" t="s">
+        <v>375</v>
+      </c>
+      <c r="H13" s="3" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A14" s="1" t="s">
         <v>48</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A14" s="1" t="s">
-        <v>49</v>
       </c>
       <c r="B14" s="1">
         <v>603</v>
@@ -2260,49 +2432,64 @@
         <v>11</v>
       </c>
       <c r="D14" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="E14" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="E14" s="1" t="s">
+      <c r="I14" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" ht="32" x14ac:dyDescent="0.2">
+      <c r="A15" s="1" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A15" s="1" t="s">
+      <c r="B15" s="1" t="s">
         <v>52</v>
-      </c>
-      <c r="B15" s="1" t="s">
-        <v>53</v>
       </c>
       <c r="C15" s="1">
         <v>4</v>
       </c>
       <c r="D15" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="E15" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="E15" s="1" t="s">
+      <c r="H15" s="4" t="s">
+        <v>384</v>
+      </c>
+      <c r="I15" t="s">
+        <v>375</v>
+      </c>
+      <c r="J15" t="s">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A16" s="1" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A16" s="1" t="s">
+      <c r="B16" s="1" t="s">
         <v>56</v>
-      </c>
-      <c r="B16" s="1" t="s">
-        <v>57</v>
       </c>
       <c r="C16" s="1">
         <v>7</v>
       </c>
       <c r="D16" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="E16" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="E16" s="1" t="s">
+      <c r="I16" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A17" s="1" t="s">
         <v>58</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A17" s="1" t="s">
-        <v>59</v>
       </c>
       <c r="B17" s="1">
         <v>603</v>
@@ -2311,35 +2498,41 @@
         <v>6</v>
       </c>
       <c r="D17" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="E17" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="E17" s="1" t="s">
+      <c r="I17" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A18" s="1" t="s">
         <v>61</v>
       </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A18" s="1" t="s">
+      <c r="B18" s="1" t="s">
         <v>62</v>
-      </c>
-      <c r="B18" s="1" t="s">
-        <v>63</v>
       </c>
       <c r="C18" s="1">
         <v>8</v>
       </c>
       <c r="D18" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="E18" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="E18" s="1" t="s">
+      <c r="I18" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A19" s="1" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A19" s="1" t="s">
+      <c r="B19" s="1" t="s">
         <v>66</v>
-      </c>
-      <c r="B19" s="1" t="s">
-        <v>67</v>
       </c>
       <c r="C19" s="1">
         <v>5</v>
@@ -2348,77 +2541,101 @@
         <v>50</v>
       </c>
       <c r="E19" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="I19" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" ht="48" x14ac:dyDescent="0.2">
+      <c r="A20" s="1" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A20" s="1" t="s">
+      <c r="B20" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="B20" s="1" t="s">
+      <c r="C20" s="1">
+        <v>1</v>
+      </c>
+      <c r="D20" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="C20" s="1">
-        <v>1</v>
-      </c>
-      <c r="D20" s="1" t="s">
+      <c r="E20" s="1" t="s">
+        <v>386</v>
+      </c>
+      <c r="F20" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="F20" s="1" t="s">
+      <c r="G20" s="1" t="s">
+        <v>375</v>
+      </c>
+      <c r="H20" s="4" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+      <c r="A21" s="1" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A21" s="1" t="s">
+      <c r="B21" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="C21" s="1">
+        <v>1</v>
+      </c>
+      <c r="D21" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="B21" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="C21" s="1">
-        <v>1</v>
-      </c>
-      <c r="D21" s="1" t="s">
+      <c r="E21" s="1" t="s">
+        <v>388</v>
+      </c>
+      <c r="F21" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="F21" s="1" t="s">
+      <c r="G21" s="1" t="s">
+        <v>375</v>
+      </c>
+      <c r="H21" s="4" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A22" s="1" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A22" s="1" t="s">
+      <c r="B22" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="B22" s="1" t="s">
+      <c r="C22" s="1">
+        <v>1</v>
+      </c>
+      <c r="D22" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="C22" s="1">
-        <v>1</v>
-      </c>
-      <c r="D22" s="1" t="s">
+      <c r="E22" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="E22" s="1" t="s">
+      <c r="I22" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A23" s="1" t="s">
         <v>79</v>
       </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A23" s="1" t="s">
+      <c r="B23" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="B23" s="1" t="s">
+      <c r="C23" s="1">
+        <v>1</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A24" s="1" t="s">
         <v>81</v>
-      </c>
-      <c r="C23" s="1">
-        <v>1</v>
-      </c>
-      <c r="D23" s="1" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A24" s="1" t="s">
-        <v>82</v>
       </c>
       <c r="B24" s="1">
         <v>603</v>
@@ -2430,12 +2647,15 @@
         <v>10</v>
       </c>
       <c r="E24" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="I24" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A25" s="1" t="s">
         <v>83</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A25" s="1" t="s">
-        <v>84</v>
       </c>
       <c r="B25" s="1">
         <v>603</v>
@@ -2444,35 +2664,41 @@
         <v>2</v>
       </c>
       <c r="D25" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="E25" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="E25" s="1" t="s">
+      <c r="I25" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A26" s="1" t="s">
         <v>86</v>
       </c>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A26" s="1" t="s">
+      <c r="B26" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="B26" s="1" t="s">
+      <c r="C26" s="1">
+        <v>1</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="E26" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="C26" s="1">
-        <v>1</v>
-      </c>
-      <c r="D26" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="E26" s="1" t="s">
+      <c r="I26" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A27" s="1" t="s">
         <v>89</v>
       </c>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A27" s="1" t="s">
+      <c r="B27" s="1" t="s">
         <v>90</v>
-      </c>
-      <c r="B27" s="1" t="s">
-        <v>91</v>
       </c>
       <c r="C27" s="1">
         <v>2</v>
@@ -2481,29 +2707,35 @@
         <v>51</v>
       </c>
       <c r="E27" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I27" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A28" s="1" t="s">
         <v>92</v>
       </c>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A28" s="1" t="s">
+      <c r="B28" s="1" t="s">
         <v>93</v>
-      </c>
-      <c r="B28" s="1" t="s">
-        <v>94</v>
       </c>
       <c r="C28" s="1">
         <v>2</v>
       </c>
       <c r="D28" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="E28" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="E28" s="1" t="s">
+      <c r="I28" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A29" s="1" t="s">
         <v>96</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A29" s="1" t="s">
-        <v>97</v>
       </c>
       <c r="B29" s="1">
         <v>603</v>
@@ -2512,18 +2744,21 @@
         <v>1</v>
       </c>
       <c r="D29" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="E29" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="E29" s="1" t="s">
+      <c r="I29" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A30" s="1" t="s">
         <v>99</v>
       </c>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A30" s="1" t="s">
+      <c r="B30" s="1" t="s">
         <v>100</v>
-      </c>
-      <c r="B30" s="1" t="s">
-        <v>101</v>
       </c>
       <c r="C30" s="1">
         <v>1</v>
@@ -2532,80 +2767,104 @@
         <v>1E-3</v>
       </c>
       <c r="E30" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="I30" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" ht="32" x14ac:dyDescent="0.2">
+      <c r="A31" s="1" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A31" s="1" t="s">
+      <c r="B31" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="B31" s="1" t="s">
+      <c r="C31" s="1">
+        <v>1</v>
+      </c>
+      <c r="D31" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="C31" s="1">
-        <v>1</v>
-      </c>
-      <c r="D31" s="1" t="s">
+      <c r="E31" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="E31" s="1" t="s">
+      <c r="G31" s="1" t="s">
+        <v>375</v>
+      </c>
+      <c r="H31" s="3" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+      <c r="A32" s="1" t="s">
         <v>106</v>
       </c>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A32" s="1" t="s">
+      <c r="B32" s="1" t="s">
         <v>107</v>
-      </c>
-      <c r="B32" s="1" t="s">
-        <v>108</v>
       </c>
       <c r="C32" s="1">
         <v>4</v>
       </c>
       <c r="D32" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="E32" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="E32" s="1" t="s">
+      <c r="H32" s="4" t="s">
+        <v>390</v>
+      </c>
+      <c r="I32" s="1" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" ht="48" x14ac:dyDescent="0.2">
+      <c r="A33" s="1" t="s">
         <v>110</v>
       </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A33" s="1" t="s">
+      <c r="B33" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="B33" s="1" t="s">
+      <c r="C33" s="1">
+        <v>1</v>
+      </c>
+      <c r="D33" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="C33" s="1">
-        <v>1</v>
-      </c>
-      <c r="D33" s="1" t="s">
+      <c r="E33" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="E33" s="1" t="s">
+      <c r="H33" s="4" t="s">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" ht="48" x14ac:dyDescent="0.2">
+      <c r="A34" s="1" t="s">
         <v>114</v>
       </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A34" s="1" t="s">
+      <c r="B34" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="B34" s="1" t="s">
+      <c r="C34" s="1">
+        <v>1</v>
+      </c>
+      <c r="D34" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="C34" s="1">
-        <v>1</v>
-      </c>
-      <c r="D34" s="1" t="s">
+      <c r="E34" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="E34" s="1" t="s">
+      <c r="H34" s="4" t="s">
+        <v>393</v>
+      </c>
+      <c r="I34" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A35" s="1" t="s">
         <v>118</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A35" s="1" t="s">
-        <v>119</v>
       </c>
       <c r="B35" s="1">
         <v>603</v>
@@ -2614,267 +2873,315 @@
         <v>2</v>
       </c>
       <c r="D35" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="E35" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="E35" s="1" t="s">
+      <c r="I35" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A36" s="1" t="s">
         <v>121</v>
       </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A36" s="1" t="s">
+      <c r="B36" s="1" t="s">
         <v>122</v>
-      </c>
-      <c r="B36" s="1" t="s">
-        <v>123</v>
       </c>
       <c r="C36" s="1">
         <v>4</v>
       </c>
       <c r="D36" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="E36" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="E36" s="1" t="s">
+      <c r="I36" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A37" s="1" t="s">
         <v>125</v>
       </c>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A37" s="1" t="s">
+      <c r="B37" s="1" t="s">
         <v>126</v>
-      </c>
-      <c r="B37" s="1" t="s">
-        <v>127</v>
       </c>
       <c r="C37" s="1">
         <v>4</v>
       </c>
       <c r="D37" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="E37" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="E37" s="1" t="s">
+      <c r="I37" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A38" s="1" t="s">
         <v>129</v>
       </c>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A38" s="1" t="s">
+      <c r="B38" s="1" t="s">
         <v>130</v>
-      </c>
-      <c r="B38" s="1" t="s">
-        <v>131</v>
       </c>
       <c r="C38" s="1">
         <v>6</v>
       </c>
       <c r="D38" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="E38" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="E38" s="1" t="s">
+      <c r="I38" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A39" s="1" t="s">
         <v>133</v>
       </c>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A39" s="1" t="s">
+      <c r="B39" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="B39" s="1" t="s">
+      <c r="C39" s="1">
+        <v>1</v>
+      </c>
+      <c r="D39" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="C39" s="1">
-        <v>1</v>
-      </c>
-      <c r="D39" s="1" t="s">
+      <c r="E39" s="1" t="s">
         <v>136</v>
       </c>
-      <c r="E39" s="1" t="s">
+      <c r="I39" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A40" s="1" t="s">
         <v>137</v>
       </c>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A40" s="1" t="s">
+      <c r="B40" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="C40" s="1">
+        <v>1</v>
+      </c>
+      <c r="D40" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="B40" s="1" t="s">
-        <v>131</v>
-      </c>
-      <c r="C40" s="1">
-        <v>1</v>
-      </c>
-      <c r="D40" s="1" t="s">
+      <c r="E40" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="I40" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A41" s="1" t="s">
         <v>139</v>
       </c>
-      <c r="E40" s="1" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A41" s="1" t="s">
+      <c r="B41" s="1" t="s">
         <v>140</v>
-      </c>
-      <c r="B41" s="1" t="s">
-        <v>141</v>
       </c>
       <c r="C41" s="1">
         <v>2</v>
       </c>
       <c r="D41" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="E41" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="E41" s="1" t="s">
+      <c r="I41" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A42" s="1" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A42" s="1" t="s">
+      <c r="B42" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C42" s="1">
+        <v>1</v>
+      </c>
+      <c r="D42" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="B42" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="C42" s="1">
-        <v>1</v>
-      </c>
-      <c r="D42" s="1" t="s">
+    </row>
+    <row r="43" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A43" s="1" t="s">
         <v>145</v>
       </c>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A43" s="1" t="s">
+      <c r="B43" s="1" t="s">
         <v>146</v>
-      </c>
-      <c r="B43" s="1" t="s">
-        <v>147</v>
       </c>
       <c r="C43" s="1">
         <v>3</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="E43" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="I43" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A44" s="1" t="s">
         <v>148</v>
       </c>
-    </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A44" s="1" t="s">
+      <c r="B44" s="1" t="s">
         <v>149</v>
-      </c>
-      <c r="B44" s="1" t="s">
-        <v>150</v>
       </c>
       <c r="C44" s="1">
         <v>2</v>
       </c>
       <c r="D44" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="E44" s="1" t="s">
         <v>151</v>
       </c>
-      <c r="E44" s="1" t="s">
+      <c r="I44" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A45" s="1" t="s">
         <v>152</v>
       </c>
-    </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A45" s="1" t="s">
+      <c r="B45" s="1" t="s">
         <v>153</v>
-      </c>
-      <c r="B45" s="1" t="s">
-        <v>154</v>
       </c>
       <c r="C45" s="1">
         <v>2</v>
       </c>
       <c r="D45" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="E45" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="E45" s="1" t="s">
+      <c r="I45" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A46" s="1" t="s">
         <v>156</v>
       </c>
-    </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A46" s="1" t="s">
+      <c r="B46" s="1" t="s">
         <v>157</v>
-      </c>
-      <c r="B46" s="1" t="s">
-        <v>158</v>
       </c>
       <c r="C46" s="1">
         <v>4</v>
       </c>
       <c r="D46" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="E46" s="1" t="s">
         <v>159</v>
       </c>
-      <c r="E46" s="1" t="s">
+      <c r="I46" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A47" s="1" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A47" s="1" t="s">
+      <c r="B47" s="1" t="s">
         <v>161</v>
-      </c>
-      <c r="B47" s="1" t="s">
-        <v>162</v>
       </c>
       <c r="C47" s="1">
         <v>2</v>
       </c>
       <c r="D47" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="E47" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="E47" s="1" t="s">
+      <c r="I47" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="48" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A48" s="1" t="s">
         <v>164</v>
       </c>
-    </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A48" s="1" t="s">
+      <c r="B48" s="1" t="s">
         <v>165</v>
       </c>
-      <c r="B48" s="1" t="s">
+      <c r="C48" s="1">
+        <v>1</v>
+      </c>
+      <c r="D48" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="E48" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="C48" s="1">
-        <v>1</v>
-      </c>
-      <c r="D48" s="1" t="s">
-        <v>120</v>
-      </c>
-      <c r="E48" s="1" t="s">
+      <c r="I48" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="49" spans="1:9" ht="32" x14ac:dyDescent="0.2">
+      <c r="A49" s="1" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A49" s="1" t="s">
+      <c r="B49" s="1" t="s">
         <v>168</v>
-      </c>
-      <c r="B49" s="1" t="s">
-        <v>169</v>
       </c>
       <c r="C49" s="1">
         <v>2</v>
       </c>
       <c r="D49" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="E49" s="1" t="s">
         <v>169</v>
       </c>
-      <c r="E49" s="1" t="s">
+      <c r="H49" s="4" t="s">
+        <v>394</v>
+      </c>
+      <c r="I49" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="50" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A50" s="1" t="s">
         <v>170</v>
       </c>
-    </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A50" s="1" t="s">
+      <c r="B50" s="1" t="s">
         <v>171</v>
-      </c>
-      <c r="B50" s="1" t="s">
-        <v>172</v>
       </c>
       <c r="C50" s="1">
         <v>5</v>
       </c>
       <c r="D50" s="1" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="E50" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="I50" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="51" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A51" s="1" t="s">
         <v>173</v>
-      </c>
-    </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A51" s="1" t="s">
-        <v>174</v>
       </c>
       <c r="B51" s="1">
         <v>603</v>
@@ -2883,49 +3190,61 @@
         <v>1</v>
       </c>
       <c r="D51" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="E51" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="E51" s="1" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="I51" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="52" spans="1:9" ht="48" x14ac:dyDescent="0.2">
       <c r="A52" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="B52" s="1" t="s">
         <v>175</v>
       </c>
-      <c r="B52" s="1" t="s">
+      <c r="C52" s="1">
+        <v>1</v>
+      </c>
+      <c r="D52" s="1" t="s">
         <v>176</v>
       </c>
-      <c r="C52" s="1">
-        <v>1</v>
-      </c>
-      <c r="D52" s="1" t="s">
+      <c r="E52" s="1" t="s">
         <v>177</v>
       </c>
-      <c r="E52" s="1" t="s">
+      <c r="H52" s="4" t="s">
+        <v>395</v>
+      </c>
+      <c r="I52" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="53" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A53" s="1" t="s">
         <v>178</v>
       </c>
-    </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A53" s="1" t="s">
-        <v>179</v>
-      </c>
       <c r="B53" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C53" s="1">
         <v>3</v>
       </c>
       <c r="D53" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="E53" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="I53" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="54" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A54" s="1" t="s">
         <v>180</v>
-      </c>
-      <c r="E53" s="1" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A54" s="1" t="s">
-        <v>181</v>
       </c>
       <c r="B54" s="1">
         <v>402</v>
@@ -2934,18 +3253,21 @@
         <v>1</v>
       </c>
       <c r="D54" s="1" t="s">
+        <v>181</v>
+      </c>
+      <c r="E54" s="1" t="s">
         <v>182</v>
       </c>
-      <c r="E54" s="1" t="s">
+      <c r="I54" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="55" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A55" s="1" t="s">
         <v>183</v>
       </c>
-    </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A55" s="1" t="s">
+      <c r="B55" s="1" t="s">
         <v>184</v>
-      </c>
-      <c r="B55" s="1" t="s">
-        <v>185</v>
       </c>
       <c r="C55" s="1">
         <v>1</v>
@@ -2954,15 +3276,18 @@
         <v>300</v>
       </c>
       <c r="E55" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="I55" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="56" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+      <c r="A56" s="1" t="s">
         <v>186</v>
       </c>
-    </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A56" s="1" t="s">
+      <c r="B56" s="1" t="s">
         <v>187</v>
-      </c>
-      <c r="B56" s="1" t="s">
-        <v>188</v>
       </c>
       <c r="C56" s="1">
         <v>4</v>
@@ -2971,46 +3296,58 @@
         <v>200</v>
       </c>
       <c r="E56" s="1" t="s">
+        <v>397</v>
+      </c>
+      <c r="H56" s="4" t="s">
+        <v>396</v>
+      </c>
+      <c r="I56" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="57" spans="1:9" ht="32" x14ac:dyDescent="0.2">
+      <c r="A57" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="B57" s="1" t="s">
         <v>189</v>
       </c>
-    </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A57" s="1" t="s">
+      <c r="C57" s="1">
+        <v>1</v>
+      </c>
+      <c r="D57" s="1" t="s">
+        <v>189</v>
+      </c>
+      <c r="F57" s="1" t="s">
         <v>190</v>
       </c>
-      <c r="B57" s="1" t="s">
+      <c r="H57" s="4" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="58" spans="1:9" ht="32" x14ac:dyDescent="0.2">
+      <c r="A58" s="1" t="s">
         <v>191</v>
       </c>
-      <c r="C57" s="1">
-        <v>1</v>
-      </c>
-      <c r="D57" s="1" t="s">
-        <v>191</v>
-      </c>
-      <c r="F57" s="1" t="s">
+      <c r="B58" s="1" t="s">
         <v>192</v>
-      </c>
-    </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A58" s="1" t="s">
-        <v>193</v>
-      </c>
-      <c r="B58" s="1" t="s">
-        <v>194</v>
       </c>
       <c r="C58" s="1">
         <v>5</v>
       </c>
       <c r="D58" s="1" t="s">
+        <v>193</v>
+      </c>
+      <c r="E58" s="1" t="s">
+        <v>194</v>
+      </c>
+      <c r="H58" s="4" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="59" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A59" s="1" t="s">
         <v>195</v>
-      </c>
-      <c r="E58" s="1" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A59" s="1" t="s">
-        <v>197</v>
       </c>
       <c r="B59" s="1">
         <v>402</v>
@@ -3019,15 +3356,18 @@
         <v>3</v>
       </c>
       <c r="D59" s="1" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="E59" s="1" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.3">
+        <v>132</v>
+      </c>
+      <c r="I59" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="60" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A60" s="1" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="B60" s="1">
         <v>402</v>
@@ -3036,40 +3376,49 @@
         <v>1</v>
       </c>
       <c r="D60" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="E60" s="1" t="s">
         <v>132</v>
       </c>
-    </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="H60" s="4" t="s">
+        <v>401</v>
+      </c>
+      <c r="I60" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="61" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A61" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="B61" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C61" s="1">
+        <v>1</v>
+      </c>
+      <c r="D61" s="1" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="62" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A62" s="1" t="s">
         <v>199</v>
       </c>
-      <c r="B61" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="C61" s="1">
-        <v>1</v>
-      </c>
-      <c r="D61" s="1" t="s">
+      <c r="B62" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C62" s="1">
+        <v>1</v>
+      </c>
+      <c r="D62" s="1" t="s">
         <v>200</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A62" s="1" t="s">
+    <row r="63" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+      <c r="A63" s="1" t="s">
         <v>201</v>
-      </c>
-      <c r="B62" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="C62" s="1">
-        <v>1</v>
-      </c>
-      <c r="D62" s="1" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A63" s="1" t="s">
-        <v>203</v>
       </c>
       <c r="B63" s="1">
         <v>402</v>
@@ -3080,887 +3429,905 @@
       <c r="D63" s="1">
         <v>100</v>
       </c>
-    </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E63" s="1" t="s">
+        <v>400</v>
+      </c>
+      <c r="H63" s="4" t="s">
+        <v>402</v>
+      </c>
+      <c r="I63" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="64" spans="1:9" ht="80" x14ac:dyDescent="0.2">
       <c r="A64" s="1" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="C64" s="1">
         <v>2</v>
       </c>
       <c r="D64" s="1" t="s">
+        <v>204</v>
+      </c>
+      <c r="E64" s="1" t="s">
+        <v>205</v>
+      </c>
+      <c r="H64" s="4" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="65" spans="1:8" ht="80" x14ac:dyDescent="0.2">
+      <c r="A65" s="1" t="s">
         <v>206</v>
       </c>
-      <c r="E64" s="1" t="s">
+      <c r="B65" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="C65" s="1">
+        <v>1</v>
+      </c>
+      <c r="D65" s="1" t="s">
         <v>207</v>
       </c>
-    </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A65" s="1" t="s">
+      <c r="E65" s="1" t="s">
+        <v>205</v>
+      </c>
+      <c r="H65" s="4" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="66" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A66" s="1" t="s">
         <v>208</v>
       </c>
-      <c r="B65" s="1" t="s">
-        <v>205</v>
-      </c>
-      <c r="C65" s="1">
-        <v>1</v>
-      </c>
-      <c r="D65" s="1" t="s">
+      <c r="B66" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C66" s="1">
+        <v>1</v>
+      </c>
+      <c r="D66" s="1" t="s">
         <v>209</v>
       </c>
-      <c r="E65" s="1" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A66" s="1" t="s">
+    </row>
+    <row r="67" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A67" s="1" t="s">
         <v>210</v>
       </c>
-      <c r="B66" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="C66" s="1">
-        <v>1</v>
-      </c>
-      <c r="D66" s="1" t="s">
+      <c r="B67" s="1" t="s">
         <v>211</v>
       </c>
-    </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A67" s="1" t="s">
+      <c r="C67" s="1">
+        <v>1</v>
+      </c>
+      <c r="D67" s="1" t="s">
         <v>212</v>
       </c>
-      <c r="B67" s="1" t="s">
+    </row>
+    <row r="68" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A68" s="1" t="s">
         <v>213</v>
       </c>
-      <c r="C67" s="1">
-        <v>1</v>
-      </c>
-      <c r="D67" s="1" t="s">
+      <c r="B68" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="C68" s="1">
+        <v>1</v>
+      </c>
+      <c r="D68" s="1" t="s">
         <v>214</v>
       </c>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A68" s="1" t="s">
+    <row r="69" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A69" s="1" t="s">
         <v>215</v>
       </c>
-      <c r="B68" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="C68" s="1">
-        <v>1</v>
-      </c>
-      <c r="D68" s="1" t="s">
+      <c r="B69" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="C69" s="1">
+        <v>1</v>
+      </c>
+      <c r="D69" s="1" t="s">
         <v>216</v>
       </c>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A69" s="1" t="s">
+    <row r="70" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A70" s="1" t="s">
         <v>217</v>
       </c>
-      <c r="B69" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="C69" s="1">
-        <v>1</v>
-      </c>
-      <c r="D69" s="1" t="s">
+      <c r="B70" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="C70" s="1">
+        <v>1</v>
+      </c>
+      <c r="D70" s="1" t="s">
         <v>218</v>
       </c>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A70" s="1" t="s">
+    <row r="71" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A71" s="1" t="s">
         <v>219</v>
       </c>
-      <c r="B70" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="C70" s="1">
-        <v>1</v>
-      </c>
-      <c r="D70" s="1" t="s">
+      <c r="B71" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="C71" s="1">
+        <v>1</v>
+      </c>
+      <c r="D71" s="1" t="s">
         <v>220</v>
       </c>
     </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A71" s="1" t="s">
+    <row r="72" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A72" s="1" t="s">
         <v>221</v>
       </c>
-      <c r="B71" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="C71" s="1">
-        <v>1</v>
-      </c>
-      <c r="D71" s="1" t="s">
+      <c r="B72" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C72" s="1">
+        <v>1</v>
+      </c>
+      <c r="D72" s="1" t="s">
         <v>222</v>
       </c>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A72" s="1" t="s">
+    <row r="73" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A73" s="1" t="s">
         <v>223</v>
       </c>
-      <c r="B72" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="C72" s="1">
-        <v>1</v>
-      </c>
-      <c r="D72" s="1" t="s">
+      <c r="B73" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="C73" s="1">
+        <v>1</v>
+      </c>
+      <c r="D73" s="1" t="s">
         <v>224</v>
       </c>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A73" s="1" t="s">
+    <row r="74" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A74" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="B73" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="C73" s="1">
-        <v>1</v>
-      </c>
-      <c r="D73" s="1" t="s">
+      <c r="B74" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C74" s="1">
+        <v>1</v>
+      </c>
+      <c r="D74" s="1" t="s">
         <v>226</v>
       </c>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A74" s="1" t="s">
+    <row r="75" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A75" s="1" t="s">
         <v>227</v>
       </c>
-      <c r="B74" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="C74" s="1">
-        <v>1</v>
-      </c>
-      <c r="D74" s="1" t="s">
+      <c r="B75" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C75" s="1">
+        <v>1</v>
+      </c>
+      <c r="D75" s="1" t="s">
         <v>228</v>
       </c>
     </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A75" s="1" t="s">
+    <row r="76" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A76" s="1" t="s">
         <v>229</v>
       </c>
-      <c r="B75" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="C75" s="1">
-        <v>1</v>
-      </c>
-      <c r="D75" s="1" t="s">
+      <c r="B76" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="C76" s="1">
+        <v>1</v>
+      </c>
+      <c r="D76" s="1" t="s">
         <v>230</v>
       </c>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A76" s="1" t="s">
+    <row r="77" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A77" s="1" t="s">
         <v>231</v>
       </c>
-      <c r="B76" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="C76" s="1">
-        <v>1</v>
-      </c>
-      <c r="D76" s="1" t="s">
+      <c r="B77" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C77" s="1">
+        <v>1</v>
+      </c>
+      <c r="D77" s="1" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A77" s="1" t="s">
+    <row r="78" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A78" s="1" t="s">
         <v>233</v>
       </c>
-      <c r="B77" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="C77" s="1">
-        <v>1</v>
-      </c>
-      <c r="D77" s="1" t="s">
+      <c r="B78" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C78" s="1">
+        <v>1</v>
+      </c>
+      <c r="D78" s="1" t="s">
         <v>234</v>
       </c>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A78" s="1" t="s">
+    <row r="79" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A79" s="1" t="s">
         <v>235</v>
       </c>
-      <c r="B78" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="C78" s="1">
-        <v>1</v>
-      </c>
-      <c r="D78" s="1" t="s">
+      <c r="B79" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="C79" s="1">
+        <v>1</v>
+      </c>
+      <c r="D79" s="1" t="s">
         <v>236</v>
       </c>
     </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A79" s="1" t="s">
+    <row r="80" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A80" s="1" t="s">
         <v>237</v>
       </c>
-      <c r="B79" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="C79" s="1">
-        <v>1</v>
-      </c>
-      <c r="D79" s="1" t="s">
+      <c r="B80" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C80" s="1">
+        <v>1</v>
+      </c>
+      <c r="D80" s="1" t="s">
         <v>238</v>
       </c>
     </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A80" s="1" t="s">
+    <row r="81" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A81" s="1" t="s">
         <v>239</v>
       </c>
-      <c r="B80" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="C80" s="1">
-        <v>1</v>
-      </c>
-      <c r="D80" s="1" t="s">
+      <c r="B81" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C81" s="1">
+        <v>1</v>
+      </c>
+      <c r="D81" s="1" t="s">
         <v>240</v>
       </c>
     </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A81" s="1" t="s">
+    <row r="82" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A82" s="1" t="s">
         <v>241</v>
       </c>
-      <c r="B81" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="C81" s="1">
-        <v>1</v>
-      </c>
-      <c r="D81" s="1" t="s">
+      <c r="B82" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C82" s="1">
+        <v>1</v>
+      </c>
+      <c r="D82" s="1" t="s">
         <v>242</v>
       </c>
     </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A82" s="1" t="s">
+    <row r="83" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A83" s="1" t="s">
         <v>243</v>
       </c>
-      <c r="B82" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="C82" s="1">
-        <v>1</v>
-      </c>
-      <c r="D82" s="1" t="s">
+      <c r="B83" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C83" s="1">
+        <v>1</v>
+      </c>
+      <c r="D83" s="1" t="s">
         <v>244</v>
       </c>
     </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A83" s="1" t="s">
+    <row r="84" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A84" s="1" t="s">
         <v>245</v>
       </c>
-      <c r="B83" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="C83" s="1">
-        <v>1</v>
-      </c>
-      <c r="D83" s="1" t="s">
+      <c r="B84" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C84" s="1">
+        <v>1</v>
+      </c>
+      <c r="D84" s="1" t="s">
         <v>246</v>
       </c>
     </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A84" s="1" t="s">
+    <row r="85" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A85" s="1" t="s">
         <v>247</v>
       </c>
-      <c r="B84" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="C84" s="1">
-        <v>1</v>
-      </c>
-      <c r="D84" s="1" t="s">
+      <c r="B85" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="C85" s="1">
+        <v>1</v>
+      </c>
+      <c r="D85" s="1" t="s">
         <v>248</v>
       </c>
     </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A85" s="1" t="s">
+    <row r="86" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A86" s="1" t="s">
         <v>249</v>
       </c>
-      <c r="B85" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="C85" s="1">
-        <v>1</v>
-      </c>
-      <c r="D85" s="1" t="s">
+      <c r="B86" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="C86" s="1">
+        <v>1</v>
+      </c>
+      <c r="D86" s="1" t="s">
         <v>250</v>
       </c>
     </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A86" s="1" t="s">
+    <row r="87" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A87" s="1" t="s">
         <v>251</v>
       </c>
-      <c r="B86" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="C86" s="1">
-        <v>1</v>
-      </c>
-      <c r="D86" s="1" t="s">
+      <c r="B87" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="C87" s="1">
+        <v>1</v>
+      </c>
+      <c r="D87" s="1" t="s">
         <v>252</v>
       </c>
     </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A87" s="1" t="s">
+    <row r="88" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A88" s="1" t="s">
         <v>253</v>
       </c>
-      <c r="B87" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="C87" s="1">
-        <v>1</v>
-      </c>
-      <c r="D87" s="1" t="s">
+      <c r="B88" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="C88" s="1">
+        <v>1</v>
+      </c>
+      <c r="D88" s="1" t="s">
         <v>254</v>
       </c>
     </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A88" s="1" t="s">
+    <row r="89" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A89" s="1" t="s">
         <v>255</v>
       </c>
-      <c r="B88" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="C88" s="1">
-        <v>1</v>
-      </c>
-      <c r="D88" s="1" t="s">
+      <c r="B89" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="C89" s="1">
+        <v>1</v>
+      </c>
+      <c r="D89" s="1" t="s">
         <v>256</v>
       </c>
     </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A89" s="1" t="s">
+    <row r="90" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A90" s="1" t="s">
         <v>257</v>
       </c>
-      <c r="B89" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="C89" s="1">
-        <v>1</v>
-      </c>
-      <c r="D89" s="1" t="s">
+      <c r="B90" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="C90" s="1">
+        <v>1</v>
+      </c>
+      <c r="D90" s="1" t="s">
         <v>258</v>
       </c>
     </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A90" s="1" t="s">
+    <row r="91" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A91" s="1" t="s">
         <v>259</v>
       </c>
-      <c r="B90" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="C90" s="1">
-        <v>1</v>
-      </c>
-      <c r="D90" s="1" t="s">
+      <c r="B91" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="C91" s="1">
+        <v>1</v>
+      </c>
+      <c r="D91" s="1" t="s">
         <v>260</v>
       </c>
     </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A91" s="1" t="s">
+    <row r="92" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A92" s="1" t="s">
         <v>261</v>
       </c>
-      <c r="B91" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="C91" s="1">
-        <v>1</v>
-      </c>
-      <c r="D91" s="1" t="s">
+      <c r="B92" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="C92" s="1">
+        <v>1</v>
+      </c>
+      <c r="D92" s="1" t="s">
         <v>262</v>
       </c>
     </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A92" s="1" t="s">
+    <row r="93" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A93" s="1" t="s">
         <v>263</v>
       </c>
-      <c r="B92" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="C92" s="1">
-        <v>1</v>
-      </c>
-      <c r="D92" s="1" t="s">
+      <c r="B93" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="C93" s="1">
+        <v>1</v>
+      </c>
+      <c r="D93" s="1" t="s">
         <v>264</v>
       </c>
     </row>
-    <row r="93" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A93" s="1" t="s">
+    <row r="94" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A94" s="1" t="s">
         <v>265</v>
       </c>
-      <c r="B93" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="C93" s="1">
-        <v>1</v>
-      </c>
-      <c r="D93" s="1" t="s">
+      <c r="B94" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C94" s="1">
+        <v>1</v>
+      </c>
+      <c r="D94" s="1" t="s">
         <v>266</v>
       </c>
     </row>
-    <row r="94" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A94" s="1" t="s">
+    <row r="95" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A95" s="1" t="s">
         <v>267</v>
       </c>
-      <c r="B94" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="C94" s="1">
-        <v>1</v>
-      </c>
-      <c r="D94" s="1" t="s">
+      <c r="B95" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="C95" s="1">
+        <v>1</v>
+      </c>
+      <c r="D95" s="1" t="s">
         <v>268</v>
       </c>
     </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A95" s="1" t="s">
+    <row r="96" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A96" s="1" t="s">
         <v>269</v>
       </c>
-      <c r="B95" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="C95" s="1">
-        <v>1</v>
-      </c>
-      <c r="D95" s="1" t="s">
+      <c r="B96" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="C96" s="1">
+        <v>1</v>
+      </c>
+      <c r="D96" s="1" t="s">
         <v>270</v>
       </c>
     </row>
-    <row r="96" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A96" s="1" t="s">
+    <row r="97" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A97" s="1" t="s">
         <v>271</v>
       </c>
-      <c r="B96" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="C96" s="1">
-        <v>1</v>
-      </c>
-      <c r="D96" s="1" t="s">
+      <c r="B97" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="C97" s="1">
+        <v>1</v>
+      </c>
+      <c r="D97" s="1" t="s">
         <v>272</v>
       </c>
     </row>
-    <row r="97" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A97" s="1" t="s">
+    <row r="98" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A98" s="1" t="s">
         <v>273</v>
       </c>
-      <c r="B97" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="C97" s="1">
-        <v>1</v>
-      </c>
-      <c r="D97" s="1" t="s">
+      <c r="B98" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="C98" s="1">
+        <v>1</v>
+      </c>
+      <c r="D98" s="1" t="s">
         <v>274</v>
       </c>
     </row>
-    <row r="98" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A98" s="1" t="s">
+    <row r="99" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A99" s="1" t="s">
         <v>275</v>
       </c>
-      <c r="B98" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="C98" s="1">
-        <v>1</v>
-      </c>
-      <c r="D98" s="1" t="s">
+      <c r="B99" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="C99" s="1">
+        <v>1</v>
+      </c>
+      <c r="D99" s="1" t="s">
         <v>276</v>
       </c>
     </row>
-    <row r="99" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A99" s="1" t="s">
+    <row r="100" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A100" s="1" t="s">
         <v>277</v>
       </c>
-      <c r="B99" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="C99" s="1">
-        <v>1</v>
-      </c>
-      <c r="D99" s="1" t="s">
+      <c r="B100" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C100" s="1">
+        <v>1</v>
+      </c>
+      <c r="D100" s="1" t="s">
         <v>278</v>
       </c>
     </row>
-    <row r="100" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A100" s="1" t="s">
+    <row r="101" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A101" s="1" t="s">
         <v>279</v>
       </c>
-      <c r="B100" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="C100" s="1">
-        <v>1</v>
-      </c>
-      <c r="D100" s="1" t="s">
+      <c r="B101" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C101" s="1">
+        <v>1</v>
+      </c>
+      <c r="D101" s="1" t="s">
         <v>280</v>
       </c>
     </row>
-    <row r="101" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A101" s="1" t="s">
+    <row r="102" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A102" s="1" t="s">
         <v>281</v>
       </c>
-      <c r="B101" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="C101" s="1">
-        <v>1</v>
-      </c>
-      <c r="D101" s="1" t="s">
+      <c r="B102" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="C102" s="1">
+        <v>1</v>
+      </c>
+      <c r="D102" s="1" t="s">
         <v>282</v>
       </c>
     </row>
-    <row r="102" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A102" s="1" t="s">
+    <row r="103" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A103" s="1" t="s">
         <v>283</v>
       </c>
-      <c r="B102" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="C102" s="1">
-        <v>1</v>
-      </c>
-      <c r="D102" s="1" t="s">
+      <c r="B103" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C103" s="1">
+        <v>1</v>
+      </c>
+      <c r="D103" s="1" t="s">
         <v>284</v>
       </c>
     </row>
-    <row r="103" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A103" s="1" t="s">
+    <row r="104" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A104" s="1" t="s">
         <v>285</v>
       </c>
-      <c r="B103" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="C103" s="1">
-        <v>1</v>
-      </c>
-      <c r="D103" s="1" t="s">
+      <c r="B104" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="C104" s="1">
+        <v>1</v>
+      </c>
+      <c r="D104" s="1" t="s">
         <v>286</v>
       </c>
     </row>
-    <row r="104" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A104" s="1" t="s">
+    <row r="105" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A105" s="1" t="s">
         <v>287</v>
       </c>
-      <c r="B104" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="C104" s="1">
-        <v>1</v>
-      </c>
-      <c r="D104" s="1" t="s">
+      <c r="B105" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="C105" s="1">
+        <v>1</v>
+      </c>
+      <c r="D105" s="1" t="s">
         <v>288</v>
       </c>
     </row>
-    <row r="105" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A105" s="1" t="s">
+    <row r="106" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A106" s="1" t="s">
         <v>289</v>
       </c>
-      <c r="B105" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="C105" s="1">
-        <v>1</v>
-      </c>
-      <c r="D105" s="1" t="s">
+      <c r="B106" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="C106" s="1">
+        <v>1</v>
+      </c>
+      <c r="D106" s="1" t="s">
         <v>290</v>
       </c>
     </row>
-    <row r="106" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A106" s="1" t="s">
+    <row r="107" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A107" s="1" t="s">
         <v>291</v>
       </c>
-      <c r="B106" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="C106" s="1">
-        <v>1</v>
-      </c>
-      <c r="D106" s="1" t="s">
+      <c r="B107" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="C107" s="1">
+        <v>1</v>
+      </c>
+      <c r="D107" s="1" t="s">
         <v>292</v>
       </c>
     </row>
-    <row r="107" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A107" s="1" t="s">
+    <row r="108" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A108" s="1" t="s">
         <v>293</v>
       </c>
-      <c r="B107" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="C107" s="1">
-        <v>1</v>
-      </c>
-      <c r="D107" s="1" t="s">
+      <c r="B108" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="C108" s="1">
+        <v>1</v>
+      </c>
+      <c r="D108" s="1" t="s">
         <v>294</v>
       </c>
     </row>
-    <row r="108" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A108" s="1" t="s">
+    <row r="109" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A109" s="1" t="s">
         <v>295</v>
       </c>
-      <c r="B108" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="C108" s="1">
-        <v>1</v>
-      </c>
-      <c r="D108" s="1" t="s">
+      <c r="B109" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="C109" s="1">
+        <v>1</v>
+      </c>
+      <c r="D109" s="1" t="s">
         <v>296</v>
       </c>
     </row>
-    <row r="109" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A109" s="1" t="s">
+    <row r="110" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A110" s="1" t="s">
         <v>297</v>
       </c>
-      <c r="B109" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="C109" s="1">
-        <v>1</v>
-      </c>
-      <c r="D109" s="1" t="s">
+      <c r="B110" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C110" s="1">
+        <v>1</v>
+      </c>
+      <c r="D110" s="1" t="s">
         <v>298</v>
       </c>
     </row>
-    <row r="110" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A110" s="1" t="s">
+    <row r="111" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A111" s="1" t="s">
         <v>299</v>
       </c>
-      <c r="B110" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="C110" s="1">
-        <v>1</v>
-      </c>
-      <c r="D110" s="1" t="s">
+      <c r="B111" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C111" s="1">
+        <v>1</v>
+      </c>
+      <c r="D111" s="1" t="s">
         <v>300</v>
       </c>
     </row>
-    <row r="111" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A111" s="1" t="s">
+    <row r="112" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A112" s="1" t="s">
         <v>301</v>
       </c>
-      <c r="B111" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="C111" s="1">
-        <v>1</v>
-      </c>
-      <c r="D111" s="1" t="s">
+      <c r="B112" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C112" s="1">
+        <v>1</v>
+      </c>
+      <c r="D112" s="1" t="s">
         <v>302</v>
       </c>
     </row>
-    <row r="112" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A112" s="1" t="s">
+    <row r="113" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A113" s="1" t="s">
         <v>303</v>
       </c>
-      <c r="B112" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="C112" s="1">
-        <v>1</v>
-      </c>
-      <c r="D112" s="1" t="s">
+      <c r="B113" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C113" s="1">
+        <v>1</v>
+      </c>
+      <c r="D113" s="1" t="s">
         <v>304</v>
       </c>
     </row>
-    <row r="113" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A113" s="1" t="s">
+    <row r="114" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A114" s="1" t="s">
         <v>305</v>
       </c>
-      <c r="B113" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="C113" s="1">
-        <v>1</v>
-      </c>
-      <c r="D113" s="1" t="s">
+      <c r="B114" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C114" s="1">
+        <v>1</v>
+      </c>
+      <c r="D114" s="1" t="s">
         <v>306</v>
       </c>
     </row>
-    <row r="114" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A114" s="1" t="s">
+    <row r="115" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A115" s="1" t="s">
         <v>307</v>
       </c>
-      <c r="B114" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="C114" s="1">
-        <v>1</v>
-      </c>
-      <c r="D114" s="1" t="s">
+      <c r="B115" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C115" s="1">
+        <v>1</v>
+      </c>
+      <c r="D115" s="1" t="s">
         <v>308</v>
       </c>
     </row>
-    <row r="115" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A115" s="1" t="s">
+    <row r="116" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A116" s="1" t="s">
         <v>309</v>
       </c>
-      <c r="B115" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="C115" s="1">
-        <v>1</v>
-      </c>
-      <c r="D115" s="1" t="s">
+      <c r="B116" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C116" s="1">
+        <v>1</v>
+      </c>
+      <c r="D116" s="1" t="s">
         <v>310</v>
       </c>
     </row>
-    <row r="116" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A116" s="1" t="s">
+    <row r="117" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A117" s="1" t="s">
         <v>311</v>
       </c>
-      <c r="B116" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="C116" s="1">
-        <v>1</v>
-      </c>
-      <c r="D116" s="1" t="s">
+      <c r="B117" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C117" s="1">
+        <v>1</v>
+      </c>
+      <c r="D117" s="1" t="s">
         <v>312</v>
       </c>
     </row>
-    <row r="117" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A117" s="1" t="s">
+    <row r="118" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A118" s="1" t="s">
         <v>313</v>
       </c>
-      <c r="B117" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="C117" s="1">
-        <v>1</v>
-      </c>
-      <c r="D117" s="1" t="s">
+      <c r="B118" s="1" t="s">
         <v>314</v>
       </c>
-    </row>
-    <row r="118" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A118" s="1" t="s">
+      <c r="C118" s="1">
+        <v>1</v>
+      </c>
+      <c r="D118" s="1" t="s">
         <v>315</v>
       </c>
-      <c r="B118" s="1" t="s">
+    </row>
+    <row r="119" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A119" s="1" t="s">
         <v>316</v>
       </c>
-      <c r="C118" s="1">
-        <v>1</v>
-      </c>
-      <c r="D118" s="1" t="s">
+      <c r="B119" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C119" s="1">
+        <v>1</v>
+      </c>
+      <c r="D119" s="1" t="s">
         <v>317</v>
       </c>
     </row>
-    <row r="119" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A119" s="1" t="s">
+    <row r="120" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A120" s="1" t="s">
         <v>318</v>
       </c>
-      <c r="B119" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="C119" s="1">
-        <v>1</v>
-      </c>
-      <c r="D119" s="1" t="s">
+      <c r="B120" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C120" s="1">
+        <v>1</v>
+      </c>
+      <c r="D120" s="1" t="s">
         <v>319</v>
       </c>
     </row>
-    <row r="120" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A120" s="1" t="s">
+    <row r="121" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A121" s="1" t="s">
         <v>320</v>
       </c>
-      <c r="B120" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="C120" s="1">
-        <v>1</v>
-      </c>
-      <c r="D120" s="1" t="s">
+      <c r="B121" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="C121" s="1">
+        <v>1</v>
+      </c>
+      <c r="D121" s="1" t="s">
         <v>321</v>
       </c>
     </row>
-    <row r="121" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A121" s="1" t="s">
+    <row r="122" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A122" s="1" t="s">
         <v>322</v>
       </c>
-      <c r="B121" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="C121" s="1">
-        <v>1</v>
-      </c>
-      <c r="D121" s="1" t="s">
+      <c r="B122" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C122" s="1">
+        <v>1</v>
+      </c>
+      <c r="D122" s="1" t="s">
         <v>323</v>
       </c>
     </row>
-    <row r="122" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A122" s="1" t="s">
+    <row r="123" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A123" s="1" t="s">
         <v>324</v>
       </c>
-      <c r="B122" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="C122" s="1">
-        <v>1</v>
-      </c>
-      <c r="D122" s="1" t="s">
+      <c r="B123" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="C123" s="1">
+        <v>1</v>
+      </c>
+      <c r="D123" s="1" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="124" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A124" s="1" t="s">
         <v>325</v>
       </c>
-    </row>
-    <row r="123" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A123" s="1" t="s">
+      <c r="B124" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="C124" s="1">
+        <v>1</v>
+      </c>
+      <c r="D124" s="1" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="125" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A125" s="1" t="s">
         <v>326</v>
       </c>
-      <c r="B123" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="C123" s="1">
-        <v>1</v>
-      </c>
-      <c r="D123" s="1" t="s">
-        <v>326</v>
-      </c>
-    </row>
-    <row r="124" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A124" s="1" t="s">
+      <c r="B125" s="1" t="s">
         <v>327</v>
-      </c>
-      <c r="B124" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="C124" s="1">
-        <v>1</v>
-      </c>
-      <c r="D124" s="1" t="s">
-        <v>327</v>
-      </c>
-    </row>
-    <row r="125" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A125" s="1" t="s">
-        <v>328</v>
-      </c>
-      <c r="B125" s="1" t="s">
-        <v>329</v>
       </c>
       <c r="C125" s="1">
         <v>3</v>
       </c>
       <c r="D125" s="1" t="s">
+        <v>328</v>
+      </c>
+      <c r="E125" s="1" t="s">
+        <v>329</v>
+      </c>
+      <c r="I125" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="126" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A126" s="1" t="s">
         <v>330</v>
-      </c>
-      <c r="E125" s="1" t="s">
-        <v>331</v>
-      </c>
-    </row>
-    <row r="126" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A126" s="1" t="s">
-        <v>332</v>
       </c>
       <c r="B126" s="1" t="s">
         <v>33</v>
@@ -3969,179 +4336,215 @@
         <v>1</v>
       </c>
       <c r="D126" s="1" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="E126" s="1" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="127" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="I126" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="127" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A127" s="1" t="s">
+        <v>332</v>
+      </c>
+      <c r="B127" s="1" t="s">
+        <v>333</v>
+      </c>
+      <c r="C127" s="1">
+        <v>1</v>
+      </c>
+      <c r="D127" s="1" t="s">
         <v>334</v>
       </c>
-      <c r="B127" s="1" t="s">
+      <c r="E127" s="1" t="s">
         <v>335</v>
       </c>
-      <c r="C127" s="1">
-        <v>1</v>
-      </c>
-      <c r="D127" s="1" t="s">
+      <c r="H127" s="1" t="s">
+        <v>404</v>
+      </c>
+      <c r="I127" s="1" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="128" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A128" s="1" t="s">
         <v>336</v>
       </c>
-      <c r="E127" s="1" t="s">
+      <c r="B128" s="1" t="s">
         <v>337</v>
       </c>
-    </row>
-    <row r="128" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A128" s="1" t="s">
+      <c r="C128" s="1">
+        <v>1</v>
+      </c>
+      <c r="D128" s="1" t="s">
         <v>338</v>
       </c>
-      <c r="B128" s="1" t="s">
+      <c r="E128" s="1" t="s">
         <v>339</v>
       </c>
-      <c r="C128" s="1">
-        <v>1</v>
-      </c>
-      <c r="D128" s="1" t="s">
+      <c r="I128" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="129" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A129" s="1" t="s">
         <v>340</v>
       </c>
-      <c r="E128" s="1" t="s">
+      <c r="B129" s="1" t="s">
         <v>341</v>
-      </c>
-    </row>
-    <row r="129" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A129" s="1" t="s">
-        <v>342</v>
-      </c>
-      <c r="B129" s="1" t="s">
-        <v>343</v>
       </c>
       <c r="C129" s="1">
         <v>3</v>
       </c>
       <c r="D129" s="1" t="s">
+        <v>341</v>
+      </c>
+      <c r="E129" s="1" t="s">
+        <v>342</v>
+      </c>
+      <c r="I129" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="130" spans="1:9" ht="64" x14ac:dyDescent="0.2">
+      <c r="A130" s="1" t="s">
         <v>343</v>
       </c>
-      <c r="E129" s="1" t="s">
+      <c r="B130" s="1" t="s">
         <v>344</v>
       </c>
-    </row>
-    <row r="130" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A130" s="1" t="s">
+      <c r="C130" s="1">
+        <v>1</v>
+      </c>
+      <c r="D130" s="1" t="s">
         <v>345</v>
       </c>
-      <c r="B130" s="1" t="s">
+      <c r="E130" s="1" t="s">
+        <v>405</v>
+      </c>
+      <c r="G130" s="1" t="s">
+        <v>375</v>
+      </c>
+      <c r="H130" s="3" t="s">
+        <v>406</v>
+      </c>
+      <c r="I130" s="1" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="131" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A131" s="1" t="s">
         <v>346</v>
       </c>
-      <c r="C130" s="1">
-        <v>1</v>
-      </c>
-      <c r="D130" s="1" t="s">
+      <c r="B131" s="1" t="s">
         <v>347</v>
       </c>
-      <c r="F130" s="1" t="s">
+      <c r="C131" s="1">
+        <v>1</v>
+      </c>
+      <c r="D131" s="1" t="s">
         <v>348</v>
       </c>
-    </row>
-    <row r="131" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A131" s="1" t="s">
+      <c r="E131" s="1" t="s">
         <v>349</v>
       </c>
-      <c r="B131" s="1" t="s">
+      <c r="I131" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="132" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A132" s="1" t="s">
         <v>350</v>
       </c>
-      <c r="C131" s="1">
-        <v>1</v>
-      </c>
-      <c r="D131" s="1" t="s">
+      <c r="B132" s="1" t="s">
         <v>351</v>
-      </c>
-      <c r="E131" s="1" t="s">
-        <v>352</v>
-      </c>
-    </row>
-    <row r="132" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A132" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="B132" s="1" t="s">
-        <v>354</v>
       </c>
       <c r="C132" s="1">
         <v>2</v>
       </c>
       <c r="D132" s="1" t="s">
+        <v>352</v>
+      </c>
+      <c r="E132" s="1" t="s">
+        <v>353</v>
+      </c>
+      <c r="I132" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="133" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A133" s="1" t="s">
+        <v>354</v>
+      </c>
+      <c r="B133" s="1" t="s">
         <v>355</v>
       </c>
-      <c r="E132" s="1" t="s">
+      <c r="C133" s="1">
+        <v>1</v>
+      </c>
+      <c r="D133" s="1" t="s">
         <v>356</v>
       </c>
-    </row>
-    <row r="133" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A133" s="1" t="s">
+      <c r="E133" s="1" t="s">
         <v>357</v>
       </c>
-      <c r="B133" s="1" t="s">
+      <c r="I133" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="134" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A134" s="1" t="s">
         <v>358</v>
       </c>
-      <c r="C133" s="1">
-        <v>1</v>
-      </c>
-      <c r="D133" s="1" t="s">
+      <c r="B134" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C134" s="1">
+        <v>1</v>
+      </c>
+      <c r="D134" s="1" t="s">
         <v>359</v>
       </c>
-      <c r="E133" s="1" t="s">
+    </row>
+    <row r="135" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A135" s="1" t="s">
         <v>360</v>
       </c>
-    </row>
-    <row r="134" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A134" s="1" t="s">
+      <c r="B135" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C135" s="1">
+        <v>1</v>
+      </c>
+      <c r="D135" s="1" t="s">
         <v>361</v>
       </c>
-      <c r="B134" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="C134" s="1">
-        <v>1</v>
-      </c>
-      <c r="D134" s="1" t="s">
+    </row>
+    <row r="136" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A136" s="1" t="s">
         <v>362</v>
       </c>
-    </row>
-    <row r="135" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A135" s="1" t="s">
+      <c r="B136" s="1" t="s">
         <v>363</v>
       </c>
-      <c r="B135" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="C135" s="1">
-        <v>1</v>
-      </c>
-      <c r="D135" s="1" t="s">
+      <c r="C136" s="1">
+        <v>1</v>
+      </c>
+      <c r="D136" s="1" t="s">
         <v>364</v>
       </c>
-    </row>
-    <row r="136" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A136" s="1" t="s">
+      <c r="E136" s="1" t="s">
         <v>365</v>
       </c>
-      <c r="B136" s="1" t="s">
+      <c r="I136" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="137" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A137" s="1" t="s">
         <v>366</v>
-      </c>
-      <c r="C136" s="1">
-        <v>1</v>
-      </c>
-      <c r="D136" s="1" t="s">
-        <v>367</v>
-      </c>
-      <c r="E136" s="1" t="s">
-        <v>368</v>
-      </c>
-    </row>
-    <row r="137" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A137" s="1" t="s">
-        <v>369</v>
       </c>
       <c r="B137" s="1">
         <v>402</v>
@@ -4150,35 +4553,41 @@
         <v>3</v>
       </c>
       <c r="D137" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E137" s="1" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="138" spans="1:6" x14ac:dyDescent="0.3">
+        <v>132</v>
+      </c>
+      <c r="I137" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="138" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A138" s="1" t="s">
+        <v>367</v>
+      </c>
+      <c r="B138" s="1" t="s">
+        <v>368</v>
+      </c>
+      <c r="C138" s="1">
+        <v>1</v>
+      </c>
+      <c r="D138" s="1" t="s">
+        <v>369</v>
+      </c>
+      <c r="E138" s="1" t="s">
         <v>370</v>
       </c>
-      <c r="B138" s="1" t="s">
+      <c r="I138" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="139" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A139" s="1" t="s">
         <v>371</v>
       </c>
-      <c r="C138" s="1">
-        <v>1</v>
-      </c>
-      <c r="D138" s="1" t="s">
+      <c r="B139" s="1" t="s">
         <v>372</v>
-      </c>
-      <c r="E138" s="1" t="s">
-        <v>373</v>
-      </c>
-    </row>
-    <row r="139" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A139" s="1" t="s">
-        <v>374</v>
-      </c>
-      <c r="B139" s="1" t="s">
-        <v>375</v>
       </c>
       <c r="C139" s="1">
         <v>1</v>
@@ -4187,10 +4596,14 @@
         <v>5</v>
       </c>
       <c r="E139" s="1" t="s">
-        <v>376</v>
+        <v>373</v>
+      </c>
+      <c r="I139" t="s">
+        <v>375</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Rushed bom review oops
</commit_message>
<xml_diff>
--- a/bom.csv.xlsx
+++ b/bom.csv.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alisruzh\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ruzha\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{D98C1871-A47A-42AA-AAE5-9A254DA12573}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C1A180E-099C-464A-858F-BA736752E69B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{EA634A8A-7489-4C3E-A3E3-2BEB5E00DD22}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{EA634A8A-7489-4C3E-A3E3-2BEB5E00DD22}"/>
   </bookViews>
   <sheets>
     <sheet name="bom" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="467" uniqueCount="377">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="646" uniqueCount="408">
   <si>
     <t>Designator</t>
   </si>
@@ -142,9 +142,6 @@
     <t>BR1</t>
   </si>
   <si>
-    <t>C14675</t>
-  </si>
-  <si>
     <t>C70, C71, C72, MCUC18</t>
   </si>
   <si>
@@ -238,18 +235,12 @@
     <t>SMF7V0A</t>
   </si>
   <si>
-    <t>SMF7V0A-E3-18-ND</t>
-  </si>
-  <si>
     <t>D2</t>
   </si>
   <si>
     <t>SMF30A</t>
   </si>
   <si>
-    <t>F5826CT-ND</t>
-  </si>
-  <si>
     <t>DC3</t>
   </si>
   <si>
@@ -331,9 +322,6 @@
     <t>C469381</t>
   </si>
   <si>
-    <t>J1</t>
-  </si>
-  <si>
     <t>3P_Pin_Header</t>
   </si>
   <si>
@@ -589,9 +577,6 @@
     <t>200_R1210</t>
   </si>
   <si>
-    <t>C26060</t>
-  </si>
-  <si>
     <t>S1</t>
   </si>
   <si>
@@ -610,9 +595,6 @@
     <t>EG1218</t>
   </si>
   <si>
-    <t>C273394</t>
-  </si>
-  <si>
     <t>SC1, SC2, XC5</t>
   </si>
   <si>
@@ -643,9 +625,6 @@
     <t>Thermistor_US</t>
   </si>
   <si>
-    <t>C2877258</t>
-  </si>
-  <si>
     <t>TH2</t>
   </si>
   <si>
@@ -1066,98 +1045,212 @@
     <t>LTC4359-DCB</t>
   </si>
   <si>
+    <t>U9</t>
+  </si>
+  <si>
+    <t>SOT-223-3_TabPin2</t>
+  </si>
+  <si>
+    <t>AMS1117-3.3</t>
+  </si>
+  <si>
+    <t>C6186</t>
+  </si>
+  <si>
+    <t>USBC1, USBC2</t>
+  </si>
+  <si>
+    <t>10uF_C0603</t>
+  </si>
+  <si>
+    <t>10 uF</t>
+  </si>
+  <si>
+    <t>C96446</t>
+  </si>
+  <si>
+    <t>USBR3</t>
+  </si>
+  <si>
+    <t>1.5k_100mW_R0603</t>
+  </si>
+  <si>
+    <t>1.5k</t>
+  </si>
+  <si>
+    <t>C22843</t>
+  </si>
+  <si>
+    <t>VCAP1TP</t>
+  </si>
+  <si>
+    <t>Vcap1TP</t>
+  </si>
+  <si>
+    <t>V_SWDTP</t>
+  </si>
+  <si>
+    <t>VSWDTP</t>
+  </si>
+  <si>
+    <t>X1</t>
+  </si>
+  <si>
+    <t>18pF_Oscillator_CRYSTAL-SMD_4P</t>
+  </si>
+  <si>
+    <t>X322516MRB4SI</t>
+  </si>
+  <si>
+    <t>C70562</t>
+  </si>
+  <si>
+    <t>XC1, XC3, XC4</t>
+  </si>
+  <si>
+    <t>XCREG1</t>
+  </si>
+  <si>
+    <t>0.47 uF_C1210</t>
+  </si>
+  <si>
+    <t>0.47 uF</t>
+  </si>
+  <si>
+    <t>C309505</t>
+  </si>
+  <si>
+    <t>XRREG1</t>
+  </si>
+  <si>
+    <t>5_1W_R2512</t>
+  </si>
+  <si>
+    <t>C5123609</t>
+  </si>
+  <si>
+    <t>Logan Flag</t>
+  </si>
+  <si>
+    <t>x</t>
+  </si>
+  <si>
+    <t>C177347</t>
+  </si>
+  <si>
+    <t>Switched</t>
+  </si>
+  <si>
+    <t>Comments</t>
+  </si>
+  <si>
+    <t>Somehow</t>
+  </si>
+  <si>
+    <t>16V, but that's okay!</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t>Validated by Logan</t>
+  </si>
+  <si>
+    <t>wrong value originally</t>
+  </si>
+  <si>
+    <t>Polarity -&gt; should make sure assigned properly</t>
+  </si>
+  <si>
+    <t>Throughhole - we can just order</t>
+  </si>
+  <si>
+    <t>C320558</t>
+  </si>
+  <si>
+    <t>Found a new tvs diode</t>
+  </si>
+  <si>
+    <t>C1973936</t>
+  </si>
+  <si>
+    <t>Found a new tvs diode - supposeely compatable with the DO-219AB package</t>
+  </si>
+  <si>
+    <t>great deal - keep pcba</t>
+  </si>
+  <si>
+    <t>This doesn't need to be PCBA - ungodly cheap tho</t>
+  </si>
+  <si>
+    <t>This doesn't need to be pcba and is smt we should buy anyway</t>
+  </si>
+  <si>
+    <t>Alisa, please double check this just cause it's complex. But looks fine</t>
+  </si>
+  <si>
+    <t>not 100% sure, but pre sure this is right</t>
+  </si>
+  <si>
+    <t>This is fine, but supposedly the same footprint as the pmos, but they look different</t>
+  </si>
+  <si>
+    <t>was - C26060 which is wrong</t>
+  </si>
+  <si>
+    <t>C102427</t>
+  </si>
+  <si>
+    <t>Throughpin all good to ignore from JLC</t>
+  </si>
+  <si>
+    <t>Not an amazing deal could do non-JLC</t>
+  </si>
+  <si>
+    <t>C4350330</t>
+  </si>
+  <si>
+    <t>Blank - Added by logan</t>
+  </si>
+  <si>
+    <t>Blank -Added by logan</t>
+  </si>
+  <si>
+    <t>Through pin and we don't necessairly want them right in the board - I would not have them assembled on board</t>
+  </si>
+  <si>
+    <t>THANK GOD THEY HAVE THIS</t>
+  </si>
+  <si>
+    <t>C7454463</t>
+  </si>
+  <si>
+    <t>I think this is the right one, pls double check505-LTC4359CDCB#TRPBFCT-ND</t>
+  </si>
+  <si>
+    <t>Place</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>DNP</t>
+  </si>
+  <si>
+    <t>J1+A31:J31</t>
+  </si>
+  <si>
+    <t>EG1903-ND</t>
+  </si>
+  <si>
     <t>505-LTC4359CDCB#TRPBFCT-ND</t>
-  </si>
-  <si>
-    <t>U9</t>
-  </si>
-  <si>
-    <t>SOT-223-3_TabPin2</t>
-  </si>
-  <si>
-    <t>AMS1117-3.3</t>
-  </si>
-  <si>
-    <t>C6186</t>
-  </si>
-  <si>
-    <t>USBC1, USBC2</t>
-  </si>
-  <si>
-    <t>10uF_C0603</t>
-  </si>
-  <si>
-    <t>10 uF</t>
-  </si>
-  <si>
-    <t>C96446</t>
-  </si>
-  <si>
-    <t>USBR3</t>
-  </si>
-  <si>
-    <t>1.5k_100mW_R0603</t>
-  </si>
-  <si>
-    <t>1.5k</t>
-  </si>
-  <si>
-    <t>C22843</t>
-  </si>
-  <si>
-    <t>VCAP1TP</t>
-  </si>
-  <si>
-    <t>Vcap1TP</t>
-  </si>
-  <si>
-    <t>V_SWDTP</t>
-  </si>
-  <si>
-    <t>VSWDTP</t>
-  </si>
-  <si>
-    <t>X1</t>
-  </si>
-  <si>
-    <t>18pF_Oscillator_CRYSTAL-SMD_4P</t>
-  </si>
-  <si>
-    <t>X322516MRB4SI</t>
-  </si>
-  <si>
-    <t>C70562</t>
-  </si>
-  <si>
-    <t>XC1, XC3, XC4</t>
-  </si>
-  <si>
-    <t>XCREG1</t>
-  </si>
-  <si>
-    <t>0.47 uF_C1210</t>
-  </si>
-  <si>
-    <t>0.47 uF</t>
-  </si>
-  <si>
-    <t>C309505</t>
-  </si>
-  <si>
-    <t>XRREG1</t>
-  </si>
-  <si>
-    <t>5_1W_R2512</t>
-  </si>
-  <si>
-    <t>C5123609</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1292,8 +1385,15 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="33">
+  <fills count="34">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1473,6 +1573,12 @@
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="10">
     <border>
@@ -1634,10 +1740,27 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="42">
@@ -1686,6 +1809,11 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FFFFCC99"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -2014,18 +2142,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2EF7A2F2-D173-446E-BAD3-537DE2CE4F10}">
-  <dimension ref="A1:F139"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:K139"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="60.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="38.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="7.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="23.77734375" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="28.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="60.453125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="38.81640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.6328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="23.81640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.36328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="28.453125" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="5.6328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.6328125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="22.6328125" style="4" customWidth="1"/>
+    <col min="10" max="10" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2044,8 +2176,20 @@
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G1" s="1" t="s">
+        <v>402</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>369</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>373</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>6</v>
       </c>
@@ -2061,8 +2205,17 @@
       <c r="E2" s="1" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G2" s="1" t="s">
+        <v>403</v>
+      </c>
+      <c r="I2" s="4" t="s">
+        <v>374</v>
+      </c>
+      <c r="J2" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>10</v>
       </c>
@@ -2078,8 +2231,14 @@
       <c r="E3" s="1" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G3" s="1" t="s">
+        <v>403</v>
+      </c>
+      <c r="J3" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>14</v>
       </c>
@@ -2095,8 +2254,14 @@
       <c r="E4" s="1" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G4" s="1" t="s">
+        <v>403</v>
+      </c>
+      <c r="J4" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>18</v>
       </c>
@@ -2112,8 +2277,14 @@
       <c r="E5" s="1" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G5" s="1" t="s">
+        <v>403</v>
+      </c>
+      <c r="J5" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>21</v>
       </c>
@@ -2129,8 +2300,17 @@
       <c r="E6" s="1" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G6" s="1" t="s">
+        <v>403</v>
+      </c>
+      <c r="I6" s="4" t="s">
+        <v>379</v>
+      </c>
+      <c r="J6" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>25</v>
       </c>
@@ -2146,8 +2326,17 @@
       <c r="F7" s="1" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G7" s="1" t="s">
+        <v>403</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>370</v>
+      </c>
+      <c r="I7" s="4" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>29</v>
       </c>
@@ -2163,8 +2352,14 @@
       <c r="E8" s="1" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G8" s="1" t="s">
+        <v>403</v>
+      </c>
+      <c r="J8" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>32</v>
       </c>
@@ -2180,8 +2375,14 @@
       <c r="E9" s="1" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G9" s="1" t="s">
+        <v>403</v>
+      </c>
+      <c r="J9" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>36</v>
       </c>
@@ -2197,8 +2398,14 @@
       <c r="E10" s="1" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G10" s="1" t="s">
+        <v>403</v>
+      </c>
+      <c r="J10" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
         <v>39</v>
       </c>
@@ -2212,46 +2419,78 @@
         <v>100</v>
       </c>
       <c r="E11" s="1" t="s">
+        <v>371</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>403</v>
+      </c>
+      <c r="H11" t="s">
+        <v>370</v>
+      </c>
+      <c r="I11" s="4" t="s">
+        <v>378</v>
+      </c>
+      <c r="J11" s="1" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A12" s="1" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A12" s="1" t="s">
+      <c r="B12" s="1" t="s">
         <v>41</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>42</v>
       </c>
       <c r="C12" s="1">
         <v>4</v>
       </c>
       <c r="D12" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="E12" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="E12" s="1" t="s">
+      <c r="G12" s="1" t="s">
+        <v>403</v>
+      </c>
+      <c r="I12" s="4" t="s">
+        <v>375</v>
+      </c>
+      <c r="J12" s="1" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" ht="29" x14ac:dyDescent="0.35">
+      <c r="A13" s="5" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A13" s="1" t="s">
+      <c r="B13" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="B13" s="1" t="s">
+      <c r="C13" s="5">
+        <v>1</v>
+      </c>
+      <c r="D13" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="C13" s="1">
-        <v>1</v>
-      </c>
-      <c r="D13" s="1" t="s">
+      <c r="E13" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="E13" s="1" t="s">
+      <c r="F13" s="5"/>
+      <c r="G13" s="5" t="s">
+        <v>404</v>
+      </c>
+      <c r="H13" s="5" t="s">
+        <v>370</v>
+      </c>
+      <c r="I13" s="6" t="s">
+        <v>386</v>
+      </c>
+      <c r="J13" s="7"/>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A14" s="1" t="s">
         <v>48</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A14" s="1" t="s">
-        <v>49</v>
       </c>
       <c r="B14" s="1">
         <v>603</v>
@@ -2260,49 +2499,73 @@
         <v>11</v>
       </c>
       <c r="D14" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="E14" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="E14" s="1" t="s">
+      <c r="G14" s="1" t="s">
+        <v>403</v>
+      </c>
+      <c r="J14" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" ht="29" x14ac:dyDescent="0.35">
+      <c r="A15" s="1" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A15" s="1" t="s">
+      <c r="B15" s="1" t="s">
         <v>52</v>
-      </c>
-      <c r="B15" s="1" t="s">
-        <v>53</v>
       </c>
       <c r="C15" s="1">
         <v>4</v>
       </c>
       <c r="D15" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="E15" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="E15" s="1" t="s">
+      <c r="G15" s="1" t="s">
+        <v>403</v>
+      </c>
+      <c r="I15" s="4" t="s">
+        <v>379</v>
+      </c>
+      <c r="J15" t="s">
+        <v>370</v>
+      </c>
+      <c r="K15" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A16" s="1" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A16" s="1" t="s">
+      <c r="B16" s="1" t="s">
         <v>56</v>
-      </c>
-      <c r="B16" s="1" t="s">
-        <v>57</v>
       </c>
       <c r="C16" s="1">
         <v>7</v>
       </c>
       <c r="D16" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="E16" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="E16" s="1" t="s">
+      <c r="G16" s="1" t="s">
+        <v>403</v>
+      </c>
+      <c r="J16" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A17" s="1" t="s">
         <v>58</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A17" s="1" t="s">
-        <v>59</v>
       </c>
       <c r="B17" s="1">
         <v>603</v>
@@ -2311,35 +2574,47 @@
         <v>6</v>
       </c>
       <c r="D17" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="E17" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="E17" s="1" t="s">
+      <c r="G17" s="1" t="s">
+        <v>403</v>
+      </c>
+      <c r="J17" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A18" s="1" t="s">
         <v>61</v>
       </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A18" s="1" t="s">
+      <c r="B18" s="1" t="s">
         <v>62</v>
-      </c>
-      <c r="B18" s="1" t="s">
-        <v>63</v>
       </c>
       <c r="C18" s="1">
         <v>8</v>
       </c>
       <c r="D18" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="E18" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="E18" s="1" t="s">
+      <c r="G18" s="1" t="s">
+        <v>403</v>
+      </c>
+      <c r="J18" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A19" s="1" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A19" s="1" t="s">
+      <c r="B19" s="1" t="s">
         <v>66</v>
-      </c>
-      <c r="B19" s="1" t="s">
-        <v>67</v>
       </c>
       <c r="C19" s="1">
         <v>5</v>
@@ -2348,77 +2623,110 @@
         <v>50</v>
       </c>
       <c r="E19" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="G19" s="1" t="s">
+        <v>403</v>
+      </c>
+      <c r="J19" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" ht="58" x14ac:dyDescent="0.35">
+      <c r="A20" s="1" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A20" s="1" t="s">
+      <c r="B20" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="B20" s="1" t="s">
+      <c r="C20" s="1">
+        <v>1</v>
+      </c>
+      <c r="D20" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="C20" s="1">
-        <v>1</v>
-      </c>
-      <c r="D20" s="1" t="s">
+      <c r="E20" s="1" t="s">
+        <v>381</v>
+      </c>
+      <c r="G20" s="1" t="s">
+        <v>403</v>
+      </c>
+      <c r="H20" s="1" t="s">
+        <v>370</v>
+      </c>
+      <c r="I20" s="4" t="s">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A21" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="F20" s="1" t="s">
+      <c r="B21" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="C21" s="1">
+        <v>1</v>
+      </c>
+      <c r="D21" s="1" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A21" s="1" t="s">
+      <c r="E21" s="1" t="s">
+        <v>383</v>
+      </c>
+      <c r="G21" s="1" t="s">
+        <v>403</v>
+      </c>
+      <c r="H21" s="1" t="s">
+        <v>370</v>
+      </c>
+      <c r="I21" s="4" t="s">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A22" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="B21" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="C21" s="1">
-        <v>1</v>
-      </c>
-      <c r="D21" s="1" t="s">
+      <c r="B22" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="F21" s="1" t="s">
+      <c r="C22" s="1">
+        <v>1</v>
+      </c>
+      <c r="D22" s="1" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A22" s="1" t="s">
+      <c r="E22" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="B22" s="1" t="s">
+      <c r="G22" s="1" t="s">
+        <v>403</v>
+      </c>
+      <c r="J22" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A23" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="C22" s="1">
-        <v>1</v>
-      </c>
-      <c r="D22" s="1" t="s">
+      <c r="B23" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="E22" s="1" t="s">
+      <c r="C23" s="1">
+        <v>1</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="G23" s="1" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A24" s="1" t="s">
         <v>79</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A23" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="B23" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="C23" s="1">
-        <v>1</v>
-      </c>
-      <c r="D23" s="1" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A24" s="1" t="s">
-        <v>82</v>
       </c>
       <c r="B24" s="1">
         <v>603</v>
@@ -2430,12 +2738,18 @@
         <v>10</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+        <v>80</v>
+      </c>
+      <c r="G24" s="1" t="s">
+        <v>403</v>
+      </c>
+      <c r="J24" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A25" s="1" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="B25" s="1">
         <v>603</v>
@@ -2444,35 +2758,47 @@
         <v>2</v>
       </c>
       <c r="D25" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="E25" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="G25" s="1" t="s">
+        <v>403</v>
+      </c>
+      <c r="J25" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A26" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="B26" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="E25" s="1" t="s">
+      <c r="C26" s="1">
+        <v>1</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="E26" s="1" t="s">
         <v>86</v>
       </c>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A26" s="1" t="s">
+      <c r="G26" s="1" t="s">
+        <v>403</v>
+      </c>
+      <c r="J26" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A27" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="B26" s="1" t="s">
+      <c r="B27" s="1" t="s">
         <v>88</v>
-      </c>
-      <c r="C26" s="1">
-        <v>1</v>
-      </c>
-      <c r="D26" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="E26" s="1" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A27" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="B27" s="1" t="s">
-        <v>91</v>
       </c>
       <c r="C27" s="1">
         <v>2</v>
@@ -2481,29 +2807,41 @@
         <v>51</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
+        <v>89</v>
+      </c>
+      <c r="G27" s="1" t="s">
+        <v>403</v>
+      </c>
+      <c r="J27" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A28" s="1" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="C28" s="1">
         <v>2</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
+        <v>93</v>
+      </c>
+      <c r="G28" s="1" t="s">
+        <v>403</v>
+      </c>
+      <c r="J28" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A29" s="1" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="B29" s="1">
         <v>603</v>
@@ -2512,18 +2850,24 @@
         <v>1</v>
       </c>
       <c r="D29" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="E29" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="G29" s="1" t="s">
+        <v>403</v>
+      </c>
+      <c r="J29" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A30" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="B30" s="1" t="s">
         <v>98</v>
-      </c>
-      <c r="E29" s="1" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A30" s="1" t="s">
-        <v>100</v>
-      </c>
-      <c r="B30" s="1" t="s">
-        <v>101</v>
       </c>
       <c r="C30" s="1">
         <v>1</v>
@@ -2532,80 +2876,121 @@
         <v>1E-3</v>
       </c>
       <c r="E30" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="G30" s="1" t="s">
+        <v>403</v>
+      </c>
+      <c r="J30" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" s="7" customFormat="1" ht="29" x14ac:dyDescent="0.35">
+      <c r="A31" s="5" t="s">
+        <v>405</v>
+      </c>
+      <c r="B31" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="C31" s="5">
+        <v>1</v>
+      </c>
+      <c r="D31" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="E31" s="5" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A31" s="1" t="s">
+      <c r="F31" s="5"/>
+      <c r="G31" s="5" t="s">
+        <v>404</v>
+      </c>
+      <c r="H31" s="5" t="s">
+        <v>370</v>
+      </c>
+      <c r="I31" s="6" t="s">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A32" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="B31" s="1" t="s">
+      <c r="B32" s="1" t="s">
         <v>104</v>
-      </c>
-      <c r="C31" s="1">
-        <v>1</v>
-      </c>
-      <c r="D31" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="E31" s="1" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A32" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="B32" s="1" t="s">
-        <v>108</v>
       </c>
       <c r="C32" s="1">
         <v>4</v>
       </c>
       <c r="D32" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="E32" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="G32" s="1" t="s">
+        <v>403</v>
+      </c>
+      <c r="I32" s="4" t="s">
+        <v>385</v>
+      </c>
+      <c r="J32" s="1" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" s="7" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A33" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="B33" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="C33" s="5">
+        <v>1</v>
+      </c>
+      <c r="D33" s="5" t="s">
         <v>109</v>
       </c>
-      <c r="E32" s="1" t="s">
+      <c r="E33" s="5" t="s">
         <v>110</v>
       </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A33" s="1" t="s">
+      <c r="F33" s="5"/>
+      <c r="G33" s="5" t="s">
+        <v>404</v>
+      </c>
+      <c r="I33" s="8" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A34" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="B33" s="1" t="s">
+      <c r="B34" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="C33" s="1">
-        <v>1</v>
-      </c>
-      <c r="D33" s="1" t="s">
+      <c r="C34" s="1">
+        <v>1</v>
+      </c>
+      <c r="D34" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="E33" s="1" t="s">
+      <c r="E34" s="1" t="s">
         <v>114</v>
       </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A34" s="1" t="s">
+      <c r="G34" s="1" t="s">
+        <v>403</v>
+      </c>
+      <c r="I34" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="J34" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A35" s="1" t="s">
         <v>115</v>
-      </c>
-      <c r="B34" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="C34" s="1">
-        <v>1</v>
-      </c>
-      <c r="D34" s="1" t="s">
-        <v>117</v>
-      </c>
-      <c r="E34" s="1" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A35" s="1" t="s">
-        <v>119</v>
       </c>
       <c r="B35" s="1">
         <v>603</v>
@@ -2614,267 +2999,363 @@
         <v>2</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
+        <v>117</v>
+      </c>
+      <c r="G35" s="1" t="s">
+        <v>403</v>
+      </c>
+      <c r="J35" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A36" s="1" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="C36" s="1">
         <v>4</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
+        <v>121</v>
+      </c>
+      <c r="G36" s="1" t="s">
+        <v>403</v>
+      </c>
+      <c r="J36" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A37" s="1" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="C37" s="1">
         <v>4</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="E37" s="1" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
+        <v>125</v>
+      </c>
+      <c r="G37" s="1" t="s">
+        <v>403</v>
+      </c>
+      <c r="J37" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A38" s="1" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="C38" s="1">
         <v>6</v>
       </c>
       <c r="D38" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="E38" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="G38" s="1" t="s">
+        <v>403</v>
+      </c>
+      <c r="J38" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="39" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A39" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="B39" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="C39" s="1">
+        <v>1</v>
+      </c>
+      <c r="D39" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="E38" s="1" t="s">
+      <c r="E39" s="1" t="s">
         <v>133</v>
       </c>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A39" s="1" t="s">
+      <c r="G39" s="1" t="s">
+        <v>403</v>
+      </c>
+      <c r="J39" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="40" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A40" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="B39" s="1" t="s">
+      <c r="B40" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="C40" s="1">
+        <v>1</v>
+      </c>
+      <c r="D40" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="C39" s="1">
-        <v>1</v>
-      </c>
-      <c r="D39" s="1" t="s">
+      <c r="E40" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="G40" s="1" t="s">
+        <v>403</v>
+      </c>
+      <c r="J40" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="41" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A41" s="1" t="s">
         <v>136</v>
       </c>
-      <c r="E39" s="1" t="s">
+      <c r="B41" s="1" t="s">
         <v>137</v>
-      </c>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A40" s="1" t="s">
-        <v>138</v>
-      </c>
-      <c r="B40" s="1" t="s">
-        <v>131</v>
-      </c>
-      <c r="C40" s="1">
-        <v>1</v>
-      </c>
-      <c r="D40" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="E40" s="1" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A41" s="1" t="s">
-        <v>140</v>
-      </c>
-      <c r="B41" s="1" t="s">
-        <v>141</v>
       </c>
       <c r="C41" s="1">
         <v>2</v>
       </c>
       <c r="D41" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="E41" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="G41" s="1" t="s">
+        <v>403</v>
+      </c>
+      <c r="J41" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="42" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A42" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="B42" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="C42" s="1">
+        <v>1</v>
+      </c>
+      <c r="D42" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="G42" s="1" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="43" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A43" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="E41" s="1" t="s">
+      <c r="B43" s="1" t="s">
         <v>143</v>
-      </c>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A42" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="B42" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="C42" s="1">
-        <v>1</v>
-      </c>
-      <c r="D42" s="1" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A43" s="1" t="s">
-        <v>146</v>
-      </c>
-      <c r="B43" s="1" t="s">
-        <v>147</v>
       </c>
       <c r="C43" s="1">
         <v>3</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="E43" s="1" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
+        <v>144</v>
+      </c>
+      <c r="G43" s="1" t="s">
+        <v>403</v>
+      </c>
+      <c r="J43" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="44" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A44" s="1" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="C44" s="1">
         <v>2</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="E44" s="1" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
+        <v>148</v>
+      </c>
+      <c r="G44" s="1" t="s">
+        <v>403</v>
+      </c>
+      <c r="J44" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="45" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A45" s="1" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="C45" s="1">
         <v>2</v>
       </c>
       <c r="D45" s="1" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="E45" s="1" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.3">
+        <v>152</v>
+      </c>
+      <c r="G45" s="1" t="s">
+        <v>403</v>
+      </c>
+      <c r="J45" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="46" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A46" s="1" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="C46" s="1">
         <v>4</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="E46" s="1" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.3">
+        <v>156</v>
+      </c>
+      <c r="G46" s="1" t="s">
+        <v>403</v>
+      </c>
+      <c r="J46" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="47" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A47" s="1" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="C47" s="1">
         <v>2</v>
       </c>
       <c r="D47" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="E47" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="G47" s="1" t="s">
+        <v>403</v>
+      </c>
+      <c r="J47" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="48" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A48" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="B48" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="C48" s="1">
+        <v>1</v>
+      </c>
+      <c r="D48" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="E48" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="E47" s="1" t="s">
+      <c r="G48" s="1" t="s">
+        <v>403</v>
+      </c>
+      <c r="J48" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="49" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+      <c r="A49" s="1" t="s">
         <v>164</v>
       </c>
-    </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A48" s="1" t="s">
+      <c r="B49" s="1" t="s">
         <v>165</v>
-      </c>
-      <c r="B48" s="1" t="s">
-        <v>166</v>
-      </c>
-      <c r="C48" s="1">
-        <v>1</v>
-      </c>
-      <c r="D48" s="1" t="s">
-        <v>120</v>
-      </c>
-      <c r="E48" s="1" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A49" s="1" t="s">
-        <v>168</v>
-      </c>
-      <c r="B49" s="1" t="s">
-        <v>169</v>
       </c>
       <c r="C49" s="1">
         <v>2</v>
       </c>
       <c r="D49" s="1" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="E49" s="1" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
+        <v>166</v>
+      </c>
+      <c r="G49" s="1" t="s">
+        <v>403</v>
+      </c>
+      <c r="I49" s="4" t="s">
+        <v>389</v>
+      </c>
+      <c r="J49" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="50" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A50" s="1" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="C50" s="1">
         <v>5</v>
       </c>
       <c r="D50" s="1" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="E50" s="1" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
+        <v>169</v>
+      </c>
+      <c r="G50" s="1" t="s">
+        <v>403</v>
+      </c>
+      <c r="J50" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="51" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A51" s="1" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="B51" s="1">
         <v>603</v>
@@ -2883,49 +3364,70 @@
         <v>1</v>
       </c>
       <c r="D51" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="E51" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="E51" s="1" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G51" s="1" t="s">
+        <v>403</v>
+      </c>
+      <c r="J51" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="52" spans="1:10" ht="58" x14ac:dyDescent="0.35">
       <c r="A52" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="B52" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="C52" s="1">
+        <v>1</v>
+      </c>
+      <c r="D52" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="E52" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="G52" s="1" t="s">
+        <v>403</v>
+      </c>
+      <c r="I52" s="4" t="s">
+        <v>390</v>
+      </c>
+      <c r="J52" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="53" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A53" s="1" t="s">
         <v>175</v>
       </c>
-      <c r="B52" s="1" t="s">
-        <v>176</v>
-      </c>
-      <c r="C52" s="1">
-        <v>1</v>
-      </c>
-      <c r="D52" s="1" t="s">
-        <v>177</v>
-      </c>
-      <c r="E52" s="1" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A53" s="1" t="s">
-        <v>179</v>
-      </c>
       <c r="B53" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C53" s="1">
         <v>3</v>
       </c>
       <c r="D53" s="1" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="E53" s="1" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.3">
+        <v>43</v>
+      </c>
+      <c r="G53" s="1" t="s">
+        <v>403</v>
+      </c>
+      <c r="J53" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="54" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A54" s="1" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="B54" s="1">
         <v>402</v>
@@ -2934,18 +3436,24 @@
         <v>1</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="E54" s="1" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.3">
+        <v>179</v>
+      </c>
+      <c r="G54" s="1" t="s">
+        <v>403</v>
+      </c>
+      <c r="J54" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="55" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A55" s="1" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="C55" s="1">
         <v>1</v>
@@ -2954,15 +3462,21 @@
         <v>300</v>
       </c>
       <c r="E55" s="1" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.3">
+        <v>182</v>
+      </c>
+      <c r="G55" s="1" t="s">
+        <v>403</v>
+      </c>
+      <c r="J55" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="56" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A56" s="1" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="C56" s="1">
         <v>4</v>
@@ -2971,46 +3485,69 @@
         <v>200</v>
       </c>
       <c r="E56" s="1" t="s">
+        <v>392</v>
+      </c>
+      <c r="G56" s="1" t="s">
+        <v>403</v>
+      </c>
+      <c r="I56" s="4" t="s">
+        <v>391</v>
+      </c>
+      <c r="J56" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="57" spans="1:10" s="7" customFormat="1" ht="29" x14ac:dyDescent="0.35">
+      <c r="A57" s="5" t="s">
+        <v>185</v>
+      </c>
+      <c r="B57" s="5" t="s">
+        <v>186</v>
+      </c>
+      <c r="C57" s="5">
+        <v>1</v>
+      </c>
+      <c r="D57" s="5" t="s">
+        <v>186</v>
+      </c>
+      <c r="E57" s="5"/>
+      <c r="F57" s="5" t="s">
+        <v>187</v>
+      </c>
+      <c r="G57" s="5" t="s">
+        <v>404</v>
+      </c>
+      <c r="I57" s="8" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="58" spans="1:10" s="7" customFormat="1" ht="29" x14ac:dyDescent="0.35">
+      <c r="A58" s="5" t="s">
+        <v>188</v>
+      </c>
+      <c r="B58" s="5" t="s">
         <v>189</v>
       </c>
-    </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A57" s="1" t="s">
+      <c r="C58" s="5">
+        <v>5</v>
+      </c>
+      <c r="D58" s="5" t="s">
         <v>190</v>
       </c>
-      <c r="B57" s="1" t="s">
+      <c r="E58" s="5"/>
+      <c r="F58" s="5" t="s">
+        <v>406</v>
+      </c>
+      <c r="G58" s="5" t="s">
+        <v>404</v>
+      </c>
+      <c r="I58" s="8" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="59" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A59" s="1" t="s">
         <v>191</v>
-      </c>
-      <c r="C57" s="1">
-        <v>1</v>
-      </c>
-      <c r="D57" s="1" t="s">
-        <v>191</v>
-      </c>
-      <c r="F57" s="1" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A58" s="1" t="s">
-        <v>193</v>
-      </c>
-      <c r="B58" s="1" t="s">
-        <v>194</v>
-      </c>
-      <c r="C58" s="1">
-        <v>5</v>
-      </c>
-      <c r="D58" s="1" t="s">
-        <v>195</v>
-      </c>
-      <c r="E58" s="1" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A59" s="1" t="s">
-        <v>197</v>
       </c>
       <c r="B59" s="1">
         <v>402</v>
@@ -3019,15 +3556,21 @@
         <v>3</v>
       </c>
       <c r="D59" s="1" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="E59" s="1" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.3">
+        <v>129</v>
+      </c>
+      <c r="G59" s="1" t="s">
+        <v>403</v>
+      </c>
+      <c r="J59" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="60" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A60" s="1" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
       <c r="B60" s="1">
         <v>402</v>
@@ -3036,40 +3579,58 @@
         <v>1</v>
       </c>
       <c r="D60" s="1" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.3">
+        <v>128</v>
+      </c>
+      <c r="E60" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="G60" s="1" t="s">
+        <v>403</v>
+      </c>
+      <c r="I60" s="4" t="s">
+        <v>396</v>
+      </c>
+      <c r="J60" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="61" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A61" s="1" t="s">
-        <v>199</v>
+        <v>193</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="C61" s="1">
         <v>1</v>
       </c>
       <c r="D61" s="1" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.3">
+        <v>194</v>
+      </c>
+      <c r="G61" s="1" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="62" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A62" s="1" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="C62" s="1">
         <v>1</v>
       </c>
       <c r="D62" s="1" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.3">
+        <v>196</v>
+      </c>
+      <c r="G62" s="1" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="63" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A63" s="1" t="s">
-        <v>203</v>
+        <v>197</v>
       </c>
       <c r="B63" s="1">
         <v>402</v>
@@ -3080,887 +3641,915 @@
       <c r="D63" s="1">
         <v>100</v>
       </c>
-    </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A64" s="1" t="s">
+      <c r="E63" s="1" t="s">
+        <v>395</v>
+      </c>
+      <c r="G63" s="1" t="s">
+        <v>403</v>
+      </c>
+      <c r="I63" s="4" t="s">
+        <v>397</v>
+      </c>
+      <c r="J63" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="64" spans="1:10" s="7" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="A64" s="5" t="s">
+        <v>198</v>
+      </c>
+      <c r="B64" s="5" t="s">
+        <v>199</v>
+      </c>
+      <c r="C64" s="5">
+        <v>2</v>
+      </c>
+      <c r="D64" s="5" t="s">
+        <v>200</v>
+      </c>
+      <c r="E64" s="5"/>
+      <c r="F64" s="5"/>
+      <c r="G64" s="5" t="s">
+        <v>404</v>
+      </c>
+      <c r="I64" s="8" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="65" spans="1:9" s="7" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="A65" s="5" t="s">
+        <v>201</v>
+      </c>
+      <c r="B65" s="5" t="s">
+        <v>199</v>
+      </c>
+      <c r="C65" s="5">
+        <v>1</v>
+      </c>
+      <c r="D65" s="5" t="s">
+        <v>202</v>
+      </c>
+      <c r="E65" s="5"/>
+      <c r="F65" s="5"/>
+      <c r="G65" s="5" t="s">
+        <v>404</v>
+      </c>
+      <c r="I65" s="8" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="66" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A66" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="B66" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="C66" s="1">
+        <v>1</v>
+      </c>
+      <c r="D66" s="1" t="s">
         <v>204</v>
       </c>
-      <c r="B64" s="1" t="s">
+    </row>
+    <row r="67" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A67" s="1" t="s">
         <v>205</v>
       </c>
-      <c r="C64" s="1">
-        <v>2</v>
-      </c>
-      <c r="D64" s="1" t="s">
+      <c r="B67" s="1" t="s">
         <v>206</v>
       </c>
-      <c r="E64" s="1" t="s">
+      <c r="C67" s="1">
+        <v>1</v>
+      </c>
+      <c r="D67" s="1" t="s">
         <v>207</v>
       </c>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A65" s="1" t="s">
+    <row r="68" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A68" s="1" t="s">
         <v>208</v>
       </c>
-      <c r="B65" s="1" t="s">
-        <v>205</v>
-      </c>
-      <c r="C65" s="1">
-        <v>1</v>
-      </c>
-      <c r="D65" s="1" t="s">
+      <c r="B68" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="C68" s="1">
+        <v>1</v>
+      </c>
+      <c r="D68" s="1" t="s">
         <v>209</v>
       </c>
-      <c r="E65" s="1" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A66" s="1" t="s">
+    </row>
+    <row r="69" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A69" s="1" t="s">
         <v>210</v>
       </c>
-      <c r="B66" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="C66" s="1">
-        <v>1</v>
-      </c>
-      <c r="D66" s="1" t="s">
+      <c r="B69" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="C69" s="1">
+        <v>1</v>
+      </c>
+      <c r="D69" s="1" t="s">
         <v>211</v>
       </c>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A67" s="1" t="s">
+    <row r="70" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A70" s="1" t="s">
         <v>212</v>
       </c>
-      <c r="B67" s="1" t="s">
+      <c r="B70" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="C70" s="1">
+        <v>1</v>
+      </c>
+      <c r="D70" s="1" t="s">
         <v>213</v>
       </c>
-      <c r="C67" s="1">
-        <v>1</v>
-      </c>
-      <c r="D67" s="1" t="s">
+    </row>
+    <row r="71" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A71" s="1" t="s">
         <v>214</v>
       </c>
-    </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A68" s="1" t="s">
+      <c r="B71" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="C71" s="1">
+        <v>1</v>
+      </c>
+      <c r="D71" s="1" t="s">
         <v>215</v>
       </c>
-      <c r="B68" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="C68" s="1">
-        <v>1</v>
-      </c>
-      <c r="D68" s="1" t="s">
+    </row>
+    <row r="72" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A72" s="1" t="s">
         <v>216</v>
       </c>
-    </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A69" s="1" t="s">
+      <c r="B72" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="C72" s="1">
+        <v>1</v>
+      </c>
+      <c r="D72" s="1" t="s">
         <v>217</v>
       </c>
-      <c r="B69" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="C69" s="1">
-        <v>1</v>
-      </c>
-      <c r="D69" s="1" t="s">
+    </row>
+    <row r="73" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A73" s="1" t="s">
         <v>218</v>
       </c>
-    </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A70" s="1" t="s">
+      <c r="B73" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="C73" s="1">
+        <v>1</v>
+      </c>
+      <c r="D73" s="1" t="s">
         <v>219</v>
       </c>
-      <c r="B70" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="C70" s="1">
-        <v>1</v>
-      </c>
-      <c r="D70" s="1" t="s">
+    </row>
+    <row r="74" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A74" s="1" t="s">
         <v>220</v>
       </c>
-    </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A71" s="1" t="s">
+      <c r="B74" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="C74" s="1">
+        <v>1</v>
+      </c>
+      <c r="D74" s="1" t="s">
         <v>221</v>
       </c>
-      <c r="B71" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="C71" s="1">
-        <v>1</v>
-      </c>
-      <c r="D71" s="1" t="s">
+    </row>
+    <row r="75" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A75" s="1" t="s">
         <v>222</v>
       </c>
-    </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A72" s="1" t="s">
+      <c r="B75" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="C75" s="1">
+        <v>1</v>
+      </c>
+      <c r="D75" s="1" t="s">
         <v>223</v>
       </c>
-      <c r="B72" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="C72" s="1">
-        <v>1</v>
-      </c>
-      <c r="D72" s="1" t="s">
+    </row>
+    <row r="76" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A76" s="1" t="s">
         <v>224</v>
       </c>
-    </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A73" s="1" t="s">
+      <c r="B76" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="C76" s="1">
+        <v>1</v>
+      </c>
+      <c r="D76" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="B73" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="C73" s="1">
-        <v>1</v>
-      </c>
-      <c r="D73" s="1" t="s">
+    </row>
+    <row r="77" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A77" s="1" t="s">
         <v>226</v>
       </c>
-    </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A74" s="1" t="s">
+      <c r="B77" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="C77" s="1">
+        <v>1</v>
+      </c>
+      <c r="D77" s="1" t="s">
         <v>227</v>
       </c>
-      <c r="B74" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="C74" s="1">
-        <v>1</v>
-      </c>
-      <c r="D74" s="1" t="s">
+    </row>
+    <row r="78" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A78" s="1" t="s">
         <v>228</v>
       </c>
-    </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A75" s="1" t="s">
+      <c r="B78" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="C78" s="1">
+        <v>1</v>
+      </c>
+      <c r="D78" s="1" t="s">
         <v>229</v>
       </c>
-      <c r="B75" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="C75" s="1">
-        <v>1</v>
-      </c>
-      <c r="D75" s="1" t="s">
+    </row>
+    <row r="79" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A79" s="1" t="s">
         <v>230</v>
       </c>
-    </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A76" s="1" t="s">
+      <c r="B79" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="C79" s="1">
+        <v>1</v>
+      </c>
+      <c r="D79" s="1" t="s">
         <v>231</v>
       </c>
-      <c r="B76" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="C76" s="1">
-        <v>1</v>
-      </c>
-      <c r="D76" s="1" t="s">
+    </row>
+    <row r="80" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A80" s="1" t="s">
         <v>232</v>
       </c>
-    </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A77" s="1" t="s">
+      <c r="B80" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="C80" s="1">
+        <v>1</v>
+      </c>
+      <c r="D80" s="1" t="s">
         <v>233</v>
       </c>
-      <c r="B77" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="C77" s="1">
-        <v>1</v>
-      </c>
-      <c r="D77" s="1" t="s">
+    </row>
+    <row r="81" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A81" s="1" t="s">
         <v>234</v>
       </c>
-    </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A78" s="1" t="s">
+      <c r="B81" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="C81" s="1">
+        <v>1</v>
+      </c>
+      <c r="D81" s="1" t="s">
         <v>235</v>
       </c>
-      <c r="B78" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="C78" s="1">
-        <v>1</v>
-      </c>
-      <c r="D78" s="1" t="s">
+    </row>
+    <row r="82" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A82" s="1" t="s">
         <v>236</v>
       </c>
-    </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A79" s="1" t="s">
+      <c r="B82" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="C82" s="1">
+        <v>1</v>
+      </c>
+      <c r="D82" s="1" t="s">
         <v>237</v>
       </c>
-      <c r="B79" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="C79" s="1">
-        <v>1</v>
-      </c>
-      <c r="D79" s="1" t="s">
+    </row>
+    <row r="83" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A83" s="1" t="s">
         <v>238</v>
       </c>
-    </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A80" s="1" t="s">
+      <c r="B83" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="C83" s="1">
+        <v>1</v>
+      </c>
+      <c r="D83" s="1" t="s">
         <v>239</v>
       </c>
-      <c r="B80" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="C80" s="1">
-        <v>1</v>
-      </c>
-      <c r="D80" s="1" t="s">
+    </row>
+    <row r="84" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A84" s="1" t="s">
         <v>240</v>
       </c>
-    </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A81" s="1" t="s">
+      <c r="B84" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="C84" s="1">
+        <v>1</v>
+      </c>
+      <c r="D84" s="1" t="s">
         <v>241</v>
       </c>
-      <c r="B81" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="C81" s="1">
-        <v>1</v>
-      </c>
-      <c r="D81" s="1" t="s">
+    </row>
+    <row r="85" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A85" s="1" t="s">
         <v>242</v>
       </c>
-    </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A82" s="1" t="s">
+      <c r="B85" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="C85" s="1">
+        <v>1</v>
+      </c>
+      <c r="D85" s="1" t="s">
         <v>243</v>
       </c>
-      <c r="B82" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="C82" s="1">
-        <v>1</v>
-      </c>
-      <c r="D82" s="1" t="s">
+    </row>
+    <row r="86" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A86" s="1" t="s">
         <v>244</v>
       </c>
-    </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A83" s="1" t="s">
+      <c r="B86" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="C86" s="1">
+        <v>1</v>
+      </c>
+      <c r="D86" s="1" t="s">
         <v>245</v>
       </c>
-      <c r="B83" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="C83" s="1">
-        <v>1</v>
-      </c>
-      <c r="D83" s="1" t="s">
+    </row>
+    <row r="87" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A87" s="1" t="s">
         <v>246</v>
       </c>
-    </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A84" s="1" t="s">
+      <c r="B87" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="C87" s="1">
+        <v>1</v>
+      </c>
+      <c r="D87" s="1" t="s">
         <v>247</v>
       </c>
-      <c r="B84" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="C84" s="1">
-        <v>1</v>
-      </c>
-      <c r="D84" s="1" t="s">
+    </row>
+    <row r="88" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A88" s="1" t="s">
         <v>248</v>
       </c>
-    </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A85" s="1" t="s">
+      <c r="B88" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="C88" s="1">
+        <v>1</v>
+      </c>
+      <c r="D88" s="1" t="s">
         <v>249</v>
       </c>
-      <c r="B85" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="C85" s="1">
-        <v>1</v>
-      </c>
-      <c r="D85" s="1" t="s">
+    </row>
+    <row r="89" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A89" s="1" t="s">
         <v>250</v>
       </c>
-    </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A86" s="1" t="s">
+      <c r="B89" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="C89" s="1">
+        <v>1</v>
+      </c>
+      <c r="D89" s="1" t="s">
         <v>251</v>
       </c>
-      <c r="B86" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="C86" s="1">
-        <v>1</v>
-      </c>
-      <c r="D86" s="1" t="s">
+    </row>
+    <row r="90" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A90" s="1" t="s">
         <v>252</v>
       </c>
-    </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A87" s="1" t="s">
+      <c r="B90" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="C90" s="1">
+        <v>1</v>
+      </c>
+      <c r="D90" s="1" t="s">
         <v>253</v>
       </c>
-      <c r="B87" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="C87" s="1">
-        <v>1</v>
-      </c>
-      <c r="D87" s="1" t="s">
+    </row>
+    <row r="91" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A91" s="1" t="s">
         <v>254</v>
       </c>
-    </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A88" s="1" t="s">
+      <c r="B91" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="C91" s="1">
+        <v>1</v>
+      </c>
+      <c r="D91" s="1" t="s">
         <v>255</v>
       </c>
-      <c r="B88" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="C88" s="1">
-        <v>1</v>
-      </c>
-      <c r="D88" s="1" t="s">
+    </row>
+    <row r="92" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A92" s="1" t="s">
         <v>256</v>
       </c>
-    </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A89" s="1" t="s">
+      <c r="B92" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="C92" s="1">
+        <v>1</v>
+      </c>
+      <c r="D92" s="1" t="s">
         <v>257</v>
       </c>
-      <c r="B89" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="C89" s="1">
-        <v>1</v>
-      </c>
-      <c r="D89" s="1" t="s">
+    </row>
+    <row r="93" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A93" s="1" t="s">
         <v>258</v>
       </c>
-    </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A90" s="1" t="s">
+      <c r="B93" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="C93" s="1">
+        <v>1</v>
+      </c>
+      <c r="D93" s="1" t="s">
         <v>259</v>
       </c>
-      <c r="B90" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="C90" s="1">
-        <v>1</v>
-      </c>
-      <c r="D90" s="1" t="s">
+    </row>
+    <row r="94" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A94" s="1" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A91" s="1" t="s">
+      <c r="B94" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="C94" s="1">
+        <v>1</v>
+      </c>
+      <c r="D94" s="1" t="s">
         <v>261</v>
       </c>
-      <c r="B91" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="C91" s="1">
-        <v>1</v>
-      </c>
-      <c r="D91" s="1" t="s">
+    </row>
+    <row r="95" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A95" s="1" t="s">
         <v>262</v>
       </c>
-    </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A92" s="1" t="s">
+      <c r="B95" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="C95" s="1">
+        <v>1</v>
+      </c>
+      <c r="D95" s="1" t="s">
         <v>263</v>
       </c>
-      <c r="B92" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="C92" s="1">
-        <v>1</v>
-      </c>
-      <c r="D92" s="1" t="s">
+    </row>
+    <row r="96" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A96" s="1" t="s">
         <v>264</v>
       </c>
-    </row>
-    <row r="93" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A93" s="1" t="s">
+      <c r="B96" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="C96" s="1">
+        <v>1</v>
+      </c>
+      <c r="D96" s="1" t="s">
         <v>265</v>
       </c>
-      <c r="B93" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="C93" s="1">
-        <v>1</v>
-      </c>
-      <c r="D93" s="1" t="s">
+    </row>
+    <row r="97" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A97" s="1" t="s">
         <v>266</v>
       </c>
-    </row>
-    <row r="94" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A94" s="1" t="s">
+      <c r="B97" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="C97" s="1">
+        <v>1</v>
+      </c>
+      <c r="D97" s="1" t="s">
         <v>267</v>
       </c>
-      <c r="B94" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="C94" s="1">
-        <v>1</v>
-      </c>
-      <c r="D94" s="1" t="s">
+    </row>
+    <row r="98" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A98" s="1" t="s">
         <v>268</v>
       </c>
-    </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A95" s="1" t="s">
+      <c r="B98" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="C98" s="1">
+        <v>1</v>
+      </c>
+      <c r="D98" s="1" t="s">
         <v>269</v>
       </c>
-      <c r="B95" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="C95" s="1">
-        <v>1</v>
-      </c>
-      <c r="D95" s="1" t="s">
+    </row>
+    <row r="99" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A99" s="1" t="s">
         <v>270</v>
       </c>
-    </row>
-    <row r="96" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A96" s="1" t="s">
+      <c r="B99" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="C99" s="1">
+        <v>1</v>
+      </c>
+      <c r="D99" s="1" t="s">
         <v>271</v>
       </c>
-      <c r="B96" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="C96" s="1">
-        <v>1</v>
-      </c>
-      <c r="D96" s="1" t="s">
+    </row>
+    <row r="100" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A100" s="1" t="s">
         <v>272</v>
       </c>
-    </row>
-    <row r="97" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A97" s="1" t="s">
+      <c r="B100" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="C100" s="1">
+        <v>1</v>
+      </c>
+      <c r="D100" s="1" t="s">
         <v>273</v>
       </c>
-      <c r="B97" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="C97" s="1">
-        <v>1</v>
-      </c>
-      <c r="D97" s="1" t="s">
+    </row>
+    <row r="101" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A101" s="1" t="s">
         <v>274</v>
       </c>
-    </row>
-    <row r="98" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A98" s="1" t="s">
+      <c r="B101" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="C101" s="1">
+        <v>1</v>
+      </c>
+      <c r="D101" s="1" t="s">
         <v>275</v>
       </c>
-      <c r="B98" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="C98" s="1">
-        <v>1</v>
-      </c>
-      <c r="D98" s="1" t="s">
+    </row>
+    <row r="102" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A102" s="1" t="s">
         <v>276</v>
       </c>
-    </row>
-    <row r="99" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A99" s="1" t="s">
+      <c r="B102" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="C102" s="1">
+        <v>1</v>
+      </c>
+      <c r="D102" s="1" t="s">
         <v>277</v>
       </c>
-      <c r="B99" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="C99" s="1">
-        <v>1</v>
-      </c>
-      <c r="D99" s="1" t="s">
+    </row>
+    <row r="103" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A103" s="1" t="s">
         <v>278</v>
       </c>
-    </row>
-    <row r="100" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A100" s="1" t="s">
+      <c r="B103" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="C103" s="1">
+        <v>1</v>
+      </c>
+      <c r="D103" s="1" t="s">
         <v>279</v>
       </c>
-      <c r="B100" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="C100" s="1">
-        <v>1</v>
-      </c>
-      <c r="D100" s="1" t="s">
+    </row>
+    <row r="104" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A104" s="1" t="s">
         <v>280</v>
       </c>
-    </row>
-    <row r="101" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A101" s="1" t="s">
+      <c r="B104" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="C104" s="1">
+        <v>1</v>
+      </c>
+      <c r="D104" s="1" t="s">
         <v>281</v>
       </c>
-      <c r="B101" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="C101" s="1">
-        <v>1</v>
-      </c>
-      <c r="D101" s="1" t="s">
+    </row>
+    <row r="105" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A105" s="1" t="s">
         <v>282</v>
       </c>
-    </row>
-    <row r="102" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A102" s="1" t="s">
+      <c r="B105" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="C105" s="1">
+        <v>1</v>
+      </c>
+      <c r="D105" s="1" t="s">
         <v>283</v>
       </c>
-      <c r="B102" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="C102" s="1">
-        <v>1</v>
-      </c>
-      <c r="D102" s="1" t="s">
+    </row>
+    <row r="106" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A106" s="1" t="s">
         <v>284</v>
       </c>
-    </row>
-    <row r="103" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A103" s="1" t="s">
+      <c r="B106" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="C106" s="1">
+        <v>1</v>
+      </c>
+      <c r="D106" s="1" t="s">
         <v>285</v>
       </c>
-      <c r="B103" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="C103" s="1">
-        <v>1</v>
-      </c>
-      <c r="D103" s="1" t="s">
+    </row>
+    <row r="107" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A107" s="1" t="s">
         <v>286</v>
       </c>
-    </row>
-    <row r="104" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A104" s="1" t="s">
+      <c r="B107" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="C107" s="1">
+        <v>1</v>
+      </c>
+      <c r="D107" s="1" t="s">
         <v>287</v>
       </c>
-      <c r="B104" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="C104" s="1">
-        <v>1</v>
-      </c>
-      <c r="D104" s="1" t="s">
+    </row>
+    <row r="108" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A108" s="1" t="s">
         <v>288</v>
       </c>
-    </row>
-    <row r="105" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A105" s="1" t="s">
+      <c r="B108" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="C108" s="1">
+        <v>1</v>
+      </c>
+      <c r="D108" s="1" t="s">
         <v>289</v>
       </c>
-      <c r="B105" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="C105" s="1">
-        <v>1</v>
-      </c>
-      <c r="D105" s="1" t="s">
+    </row>
+    <row r="109" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A109" s="1" t="s">
         <v>290</v>
       </c>
-    </row>
-    <row r="106" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A106" s="1" t="s">
+      <c r="B109" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="C109" s="1">
+        <v>1</v>
+      </c>
+      <c r="D109" s="1" t="s">
         <v>291</v>
       </c>
-      <c r="B106" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="C106" s="1">
-        <v>1</v>
-      </c>
-      <c r="D106" s="1" t="s">
+    </row>
+    <row r="110" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A110" s="1" t="s">
         <v>292</v>
       </c>
-    </row>
-    <row r="107" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A107" s="1" t="s">
+      <c r="B110" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="C110" s="1">
+        <v>1</v>
+      </c>
+      <c r="D110" s="1" t="s">
         <v>293</v>
       </c>
-      <c r="B107" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="C107" s="1">
-        <v>1</v>
-      </c>
-      <c r="D107" s="1" t="s">
+    </row>
+    <row r="111" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A111" s="1" t="s">
         <v>294</v>
       </c>
-    </row>
-    <row r="108" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A108" s="1" t="s">
+      <c r="B111" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="C111" s="1">
+        <v>1</v>
+      </c>
+      <c r="D111" s="1" t="s">
         <v>295</v>
       </c>
-      <c r="B108" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="C108" s="1">
-        <v>1</v>
-      </c>
-      <c r="D108" s="1" t="s">
+    </row>
+    <row r="112" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A112" s="1" t="s">
         <v>296</v>
       </c>
-    </row>
-    <row r="109" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A109" s="1" t="s">
+      <c r="B112" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="C112" s="1">
+        <v>1</v>
+      </c>
+      <c r="D112" s="1" t="s">
         <v>297</v>
       </c>
-      <c r="B109" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="C109" s="1">
-        <v>1</v>
-      </c>
-      <c r="D109" s="1" t="s">
+    </row>
+    <row r="113" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A113" s="1" t="s">
         <v>298</v>
       </c>
-    </row>
-    <row r="110" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A110" s="1" t="s">
+      <c r="B113" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="C113" s="1">
+        <v>1</v>
+      </c>
+      <c r="D113" s="1" t="s">
         <v>299</v>
       </c>
-      <c r="B110" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="C110" s="1">
-        <v>1</v>
-      </c>
-      <c r="D110" s="1" t="s">
+    </row>
+    <row r="114" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A114" s="1" t="s">
         <v>300</v>
       </c>
-    </row>
-    <row r="111" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A111" s="1" t="s">
+      <c r="B114" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="C114" s="1">
+        <v>1</v>
+      </c>
+      <c r="D114" s="1" t="s">
         <v>301</v>
       </c>
-      <c r="B111" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="C111" s="1">
-        <v>1</v>
-      </c>
-      <c r="D111" s="1" t="s">
+    </row>
+    <row r="115" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A115" s="1" t="s">
         <v>302</v>
       </c>
-    </row>
-    <row r="112" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A112" s="1" t="s">
+      <c r="B115" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="C115" s="1">
+        <v>1</v>
+      </c>
+      <c r="D115" s="1" t="s">
         <v>303</v>
       </c>
-      <c r="B112" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="C112" s="1">
-        <v>1</v>
-      </c>
-      <c r="D112" s="1" t="s">
+    </row>
+    <row r="116" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A116" s="1" t="s">
         <v>304</v>
       </c>
-    </row>
-    <row r="113" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A113" s="1" t="s">
+      <c r="B116" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="C116" s="1">
+        <v>1</v>
+      </c>
+      <c r="D116" s="1" t="s">
         <v>305</v>
       </c>
-      <c r="B113" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="C113" s="1">
-        <v>1</v>
-      </c>
-      <c r="D113" s="1" t="s">
+    </row>
+    <row r="117" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A117" s="1" t="s">
         <v>306</v>
       </c>
-    </row>
-    <row r="114" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A114" s="1" t="s">
+      <c r="B117" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="C117" s="1">
+        <v>1</v>
+      </c>
+      <c r="D117" s="1" t="s">
         <v>307</v>
       </c>
-      <c r="B114" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="C114" s="1">
-        <v>1</v>
-      </c>
-      <c r="D114" s="1" t="s">
+    </row>
+    <row r="118" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A118" s="1" t="s">
         <v>308</v>
       </c>
-    </row>
-    <row r="115" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A115" s="1" t="s">
+      <c r="B118" s="1" t="s">
         <v>309</v>
       </c>
-      <c r="B115" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="C115" s="1">
-        <v>1</v>
-      </c>
-      <c r="D115" s="1" t="s">
+      <c r="C118" s="1">
+        <v>1</v>
+      </c>
+      <c r="D118" s="1" t="s">
         <v>310</v>
       </c>
     </row>
-    <row r="116" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A116" s="1" t="s">
+    <row r="119" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A119" s="1" t="s">
         <v>311</v>
       </c>
-      <c r="B116" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="C116" s="1">
-        <v>1</v>
-      </c>
-      <c r="D116" s="1" t="s">
+      <c r="B119" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="C119" s="1">
+        <v>1</v>
+      </c>
+      <c r="D119" s="1" t="s">
         <v>312</v>
       </c>
     </row>
-    <row r="117" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A117" s="1" t="s">
+    <row r="120" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A120" s="1" t="s">
         <v>313</v>
       </c>
-      <c r="B117" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="C117" s="1">
-        <v>1</v>
-      </c>
-      <c r="D117" s="1" t="s">
+      <c r="B120" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="C120" s="1">
+        <v>1</v>
+      </c>
+      <c r="D120" s="1" t="s">
         <v>314</v>
       </c>
     </row>
-    <row r="118" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A118" s="1" t="s">
+    <row r="121" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A121" s="1" t="s">
         <v>315</v>
       </c>
-      <c r="B118" s="1" t="s">
+      <c r="B121" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="C121" s="1">
+        <v>1</v>
+      </c>
+      <c r="D121" s="1" t="s">
         <v>316</v>
       </c>
-      <c r="C118" s="1">
-        <v>1</v>
-      </c>
-      <c r="D118" s="1" t="s">
+    </row>
+    <row r="122" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A122" s="1" t="s">
         <v>317</v>
       </c>
-    </row>
-    <row r="119" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A119" s="1" t="s">
+      <c r="B122" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="C122" s="1">
+        <v>1</v>
+      </c>
+      <c r="D122" s="1" t="s">
         <v>318</v>
       </c>
-      <c r="B119" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="C119" s="1">
-        <v>1</v>
-      </c>
-      <c r="D119" s="1" t="s">
+    </row>
+    <row r="123" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A123" s="1" t="s">
         <v>319</v>
       </c>
-    </row>
-    <row r="120" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A120" s="1" t="s">
+      <c r="B123" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="C123" s="1">
+        <v>1</v>
+      </c>
+      <c r="D123" s="1" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="124" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A124" s="1" t="s">
         <v>320</v>
       </c>
-      <c r="B120" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="C120" s="1">
-        <v>1</v>
-      </c>
-      <c r="D120" s="1" t="s">
+      <c r="B124" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="C124" s="1">
+        <v>1</v>
+      </c>
+      <c r="D124" s="1" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="125" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A125" s="1" t="s">
         <v>321</v>
       </c>
-    </row>
-    <row r="121" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A121" s="1" t="s">
+      <c r="B125" s="1" t="s">
         <v>322</v>
-      </c>
-      <c r="B121" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="C121" s="1">
-        <v>1</v>
-      </c>
-      <c r="D121" s="1" t="s">
-        <v>323</v>
-      </c>
-    </row>
-    <row r="122" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A122" s="1" t="s">
-        <v>324</v>
-      </c>
-      <c r="B122" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="C122" s="1">
-        <v>1</v>
-      </c>
-      <c r="D122" s="1" t="s">
-        <v>325</v>
-      </c>
-    </row>
-    <row r="123" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A123" s="1" t="s">
-        <v>326</v>
-      </c>
-      <c r="B123" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="C123" s="1">
-        <v>1</v>
-      </c>
-      <c r="D123" s="1" t="s">
-        <v>326</v>
-      </c>
-    </row>
-    <row r="124" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A124" s="1" t="s">
-        <v>327</v>
-      </c>
-      <c r="B124" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="C124" s="1">
-        <v>1</v>
-      </c>
-      <c r="D124" s="1" t="s">
-        <v>327</v>
-      </c>
-    </row>
-    <row r="125" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A125" s="1" t="s">
-        <v>328</v>
-      </c>
-      <c r="B125" s="1" t="s">
-        <v>329</v>
       </c>
       <c r="C125" s="1">
         <v>3</v>
       </c>
       <c r="D125" s="1" t="s">
-        <v>330</v>
+        <v>323</v>
       </c>
       <c r="E125" s="1" t="s">
-        <v>331</v>
-      </c>
-    </row>
-    <row r="126" spans="1:5" x14ac:dyDescent="0.3">
+        <v>324</v>
+      </c>
+      <c r="G125" s="1" t="s">
+        <v>403</v>
+      </c>
+      <c r="J125" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="126" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A126" s="1" t="s">
-        <v>332</v>
+        <v>325</v>
       </c>
       <c r="B126" s="1" t="s">
         <v>33</v>
@@ -3969,179 +4558,251 @@
         <v>1</v>
       </c>
       <c r="D126" s="1" t="s">
-        <v>333</v>
+        <v>326</v>
       </c>
       <c r="E126" s="1" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="127" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G126" s="1" t="s">
+        <v>403</v>
+      </c>
+      <c r="J126" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="127" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A127" s="1" t="s">
+        <v>327</v>
+      </c>
+      <c r="B127" s="1" t="s">
+        <v>328</v>
+      </c>
+      <c r="C127" s="1">
+        <v>1</v>
+      </c>
+      <c r="D127" s="1" t="s">
+        <v>329</v>
+      </c>
+      <c r="E127" s="1" t="s">
+        <v>330</v>
+      </c>
+      <c r="G127" s="1" t="s">
+        <v>403</v>
+      </c>
+      <c r="I127" s="1" t="s">
+        <v>399</v>
+      </c>
+      <c r="J127" s="1" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="128" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A128" s="1" t="s">
+        <v>331</v>
+      </c>
+      <c r="B128" s="1" t="s">
+        <v>332</v>
+      </c>
+      <c r="C128" s="1">
+        <v>1</v>
+      </c>
+      <c r="D128" s="1" t="s">
+        <v>333</v>
+      </c>
+      <c r="E128" s="1" t="s">
         <v>334</v>
       </c>
-      <c r="B127" s="1" t="s">
+      <c r="G128" s="1" t="s">
+        <v>403</v>
+      </c>
+      <c r="J128" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="129" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A129" s="1" t="s">
         <v>335</v>
       </c>
-      <c r="C127" s="1">
-        <v>1</v>
-      </c>
-      <c r="D127" s="1" t="s">
+      <c r="B129" s="1" t="s">
         <v>336</v>
-      </c>
-      <c r="E127" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="128" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A128" s="1" t="s">
-        <v>338</v>
-      </c>
-      <c r="B128" s="1" t="s">
-        <v>339</v>
-      </c>
-      <c r="C128" s="1">
-        <v>1</v>
-      </c>
-      <c r="D128" s="1" t="s">
-        <v>340</v>
-      </c>
-      <c r="E128" s="1" t="s">
-        <v>341</v>
-      </c>
-    </row>
-    <row r="129" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A129" s="1" t="s">
-        <v>342</v>
-      </c>
-      <c r="B129" s="1" t="s">
-        <v>343</v>
       </c>
       <c r="C129" s="1">
         <v>3</v>
       </c>
       <c r="D129" s="1" t="s">
+        <v>336</v>
+      </c>
+      <c r="E129" s="1" t="s">
+        <v>337</v>
+      </c>
+      <c r="G129" s="1" t="s">
+        <v>403</v>
+      </c>
+      <c r="J129" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="130" spans="1:10" s="7" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+      <c r="A130" s="5" t="s">
+        <v>338</v>
+      </c>
+      <c r="B130" s="5" t="s">
+        <v>339</v>
+      </c>
+      <c r="C130" s="5">
+        <v>1</v>
+      </c>
+      <c r="D130" s="5" t="s">
+        <v>340</v>
+      </c>
+      <c r="E130" s="5" t="s">
+        <v>400</v>
+      </c>
+      <c r="F130" s="5" t="s">
+        <v>407</v>
+      </c>
+      <c r="G130" s="5" t="s">
+        <v>404</v>
+      </c>
+      <c r="H130" s="5" t="s">
+        <v>370</v>
+      </c>
+      <c r="I130" s="6" t="s">
+        <v>401</v>
+      </c>
+      <c r="J130" s="5" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="131" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A131" s="1" t="s">
+        <v>341</v>
+      </c>
+      <c r="B131" s="1" t="s">
+        <v>342</v>
+      </c>
+      <c r="C131" s="1">
+        <v>1</v>
+      </c>
+      <c r="D131" s="1" t="s">
         <v>343</v>
       </c>
-      <c r="E129" s="1" t="s">
+      <c r="E131" s="1" t="s">
         <v>344</v>
       </c>
-    </row>
-    <row r="130" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A130" s="1" t="s">
+      <c r="G131" s="1" t="s">
+        <v>403</v>
+      </c>
+      <c r="J131" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="132" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A132" s="1" t="s">
         <v>345</v>
       </c>
-      <c r="B130" s="1" t="s">
+      <c r="B132" s="1" t="s">
         <v>346</v>
-      </c>
-      <c r="C130" s="1">
-        <v>1</v>
-      </c>
-      <c r="D130" s="1" t="s">
-        <v>347</v>
-      </c>
-      <c r="F130" s="1" t="s">
-        <v>348</v>
-      </c>
-    </row>
-    <row r="131" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A131" s="1" t="s">
-        <v>349</v>
-      </c>
-      <c r="B131" s="1" t="s">
-        <v>350</v>
-      </c>
-      <c r="C131" s="1">
-        <v>1</v>
-      </c>
-      <c r="D131" s="1" t="s">
-        <v>351</v>
-      </c>
-      <c r="E131" s="1" t="s">
-        <v>352</v>
-      </c>
-    </row>
-    <row r="132" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A132" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="B132" s="1" t="s">
-        <v>354</v>
       </c>
       <c r="C132" s="1">
         <v>2</v>
       </c>
       <c r="D132" s="1" t="s">
+        <v>347</v>
+      </c>
+      <c r="E132" s="1" t="s">
+        <v>348</v>
+      </c>
+      <c r="G132" s="1" t="s">
+        <v>403</v>
+      </c>
+      <c r="J132" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="133" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A133" s="1" t="s">
+        <v>349</v>
+      </c>
+      <c r="B133" s="1" t="s">
+        <v>350</v>
+      </c>
+      <c r="C133" s="1">
+        <v>1</v>
+      </c>
+      <c r="D133" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="E133" s="1" t="s">
+        <v>352</v>
+      </c>
+      <c r="G133" s="1" t="s">
+        <v>403</v>
+      </c>
+      <c r="J133" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="134" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A134" s="1" t="s">
+        <v>353</v>
+      </c>
+      <c r="B134" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="C134" s="1">
+        <v>1</v>
+      </c>
+      <c r="D134" s="1" t="s">
+        <v>354</v>
+      </c>
+      <c r="G134" s="1" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="135" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A135" s="1" t="s">
         <v>355</v>
       </c>
-      <c r="E132" s="1" t="s">
+      <c r="B135" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="C135" s="1">
+        <v>1</v>
+      </c>
+      <c r="D135" s="1" t="s">
         <v>356</v>
       </c>
-    </row>
-    <row r="133" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A133" s="1" t="s">
+      <c r="G135" s="1" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="136" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A136" s="1" t="s">
         <v>357</v>
       </c>
-      <c r="B133" s="1" t="s">
+      <c r="B136" s="1" t="s">
         <v>358</v>
       </c>
-      <c r="C133" s="1">
-        <v>1</v>
-      </c>
-      <c r="D133" s="1" t="s">
+      <c r="C136" s="1">
+        <v>1</v>
+      </c>
+      <c r="D136" s="1" t="s">
         <v>359</v>
       </c>
-      <c r="E133" s="1" t="s">
+      <c r="E136" s="1" t="s">
         <v>360</v>
       </c>
-    </row>
-    <row r="134" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A134" s="1" t="s">
+      <c r="G136" s="1" t="s">
+        <v>403</v>
+      </c>
+      <c r="J136" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="137" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A137" s="1" t="s">
         <v>361</v>
-      </c>
-      <c r="B134" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="C134" s="1">
-        <v>1</v>
-      </c>
-      <c r="D134" s="1" t="s">
-        <v>362</v>
-      </c>
-    </row>
-    <row r="135" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A135" s="1" t="s">
-        <v>363</v>
-      </c>
-      <c r="B135" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="C135" s="1">
-        <v>1</v>
-      </c>
-      <c r="D135" s="1" t="s">
-        <v>364</v>
-      </c>
-    </row>
-    <row r="136" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A136" s="1" t="s">
-        <v>365</v>
-      </c>
-      <c r="B136" s="1" t="s">
-        <v>366</v>
-      </c>
-      <c r="C136" s="1">
-        <v>1</v>
-      </c>
-      <c r="D136" s="1" t="s">
-        <v>367</v>
-      </c>
-      <c r="E136" s="1" t="s">
-        <v>368</v>
-      </c>
-    </row>
-    <row r="137" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A137" s="1" t="s">
-        <v>369</v>
       </c>
       <c r="B137" s="1">
         <v>402</v>
@@ -4150,35 +4811,47 @@
         <v>3</v>
       </c>
       <c r="D137" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E137" s="1" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="138" spans="1:6" x14ac:dyDescent="0.3">
+        <v>129</v>
+      </c>
+      <c r="G137" s="1" t="s">
+        <v>403</v>
+      </c>
+      <c r="J137" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="138" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A138" s="1" t="s">
-        <v>370</v>
+        <v>362</v>
       </c>
       <c r="B138" s="1" t="s">
-        <v>371</v>
+        <v>363</v>
       </c>
       <c r="C138" s="1">
         <v>1</v>
       </c>
       <c r="D138" s="1" t="s">
-        <v>372</v>
+        <v>364</v>
       </c>
       <c r="E138" s="1" t="s">
-        <v>373</v>
-      </c>
-    </row>
-    <row r="139" spans="1:6" x14ac:dyDescent="0.3">
+        <v>365</v>
+      </c>
+      <c r="G138" s="1" t="s">
+        <v>403</v>
+      </c>
+      <c r="J138" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="139" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A139" s="1" t="s">
-        <v>374</v>
+        <v>366</v>
       </c>
       <c r="B139" s="1" t="s">
-        <v>375</v>
+        <v>367</v>
       </c>
       <c r="C139" s="1">
         <v>1</v>
@@ -4187,10 +4860,17 @@
         <v>5</v>
       </c>
       <c r="E139" s="1" t="s">
-        <v>376</v>
+        <v>368</v>
+      </c>
+      <c r="G139" s="1" t="s">
+        <v>403</v>
+      </c>
+      <c r="J139" t="s">
+        <v>370</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
</xml_diff>